<commit_message>
Follow-ups 16-18: web gap fill, Excel COM audit, share-count fix
WS16 filled the consensus gaps from Chrome (2Q24 next-quarter Street $3.84bn;
Zacks ADR consensus for five prints), re-attributed five print reactions to
guidance, withdrew two red-team corrections, and logged post-5-Sep news.
WS17 recalculated the workbook in Excel 16 via COM (0 error cells, 2,348
formulas matching Python), fixed an inert scenario selector and 121 literal
constants, and found the 1H26 buyback double-counted in the share roll.
WS18 fixed the share roll in both the Python mirror and the Excel builder
(FY26E shares 580.3M -> 588.9M), regenerated the model, re-ran the audit
(216/216 outputs, 143/143 scenario checks), and updated the synthesis: base
football-field mean $160, bear $76, bull $233.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LzKWHQs6AMpQWUKvHPXdBh
</commit_message>
<xml_diff>
--- a/model/ABNB_driver_model.xlsx
+++ b/model/ABNB_driver_model.xlsx
@@ -136,7 +136,7 @@
     <xf numFmtId="166" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -526,7 +526,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Overnight run 6-7 Sep 2026 (workstream 13). Yellow cells are inputs; everything downstream is a live formula. Sources name the workstream that supplied the value.</t>
+          <t>Overnight run 6-7 Sep 2026 (workstream 13). Yellow cells are inputs; everything downstream is a live formula. The other hard numbers in the file are the History actuals table, the external Street / Card bars (each with its vendor and date) and the Recon sheet's Python-mirror column. Sources name the workstream that supplied the value.</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Drives the headline blocks on Valuation and Card_5Nov. All three scenarios are computed in full on Revenue / Costs / Cash.</t>
+          <t>Drives the Active column here and the Active column on Valuation (sections 1-4) and Card_5Nov. All three scenarios are computed in full on Revenue / Costs / Cash, so the Bear / Base / Bull columns never move when this cell changes.</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>5 Sep reverse-DCF convention: 10-year fade to terminal</t>
+          <t>5 Sep reverse-DCF convention: 10-year fade to terminal. LAYOUT-FIXED: the DCF grid on Valuation section 3 is ten written-out rows, so changing this cell does not resize the grid and has no effect on any output</t>
         </is>
       </c>
     </row>
@@ -3109,7 +3109,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>pp</t>
+          <t>y/y</t>
         </is>
       </c>
       <c r="C95" s="10" t="n">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>WS07: no FX view three years out; zero in every case so FX does not flatter the path</t>
+          <t>WS07: no FX view three years out; zero in every case so FX does not flatter the path. UNIT: a fraction, percent-formatted (0.015 = +1.5pp), NOT the plain percentage-point number used by the quarterly FX rows in section C</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>pp</t>
+          <t>y/y</t>
         </is>
       </c>
       <c r="C96" s="10" t="n">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>same</t>
+          <t>same; a fraction, percent-formatted, not a percentage-point number</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X103"/>
+  <dimension ref="A1:X118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7265,23 +7265,27 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>3Q25 nights (M)</t>
+          <t>1H2026 SBC ($M)</t>
         </is>
       </c>
       <c r="B50" s="15">
-        <f>B23</f>
-        <v/>
-      </c>
-      <c r="C50" s="2" t="inlineStr"/>
+        <f>I25+I26</f>
+        <v/>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>actual; used by the 2H26 share roll</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>3Q25 GBV ($M)</t>
+          <t>3Q25 nights (M)</t>
         </is>
       </c>
       <c r="B51" s="15">
-        <f>C23</f>
+        <f>B23</f>
         <v/>
       </c>
       <c r="C51" s="2" t="inlineStr"/>
@@ -7289,11 +7293,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>3Q25 ADR ($)</t>
-        </is>
-      </c>
-      <c r="B52" s="9">
-        <f>D23</f>
+          <t>3Q25 GBV ($M)</t>
+        </is>
+      </c>
+      <c r="B52" s="15">
+        <f>C23</f>
         <v/>
       </c>
       <c r="C52" s="2" t="inlineStr"/>
@@ -7301,11 +7305,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>3Q25 revenue ($M)</t>
-        </is>
-      </c>
-      <c r="B53" s="15">
-        <f>E23</f>
+          <t>3Q25 ADR ($)</t>
+        </is>
+      </c>
+      <c r="B53" s="9">
+        <f>D23</f>
         <v/>
       </c>
       <c r="C53" s="2" t="inlineStr"/>
@@ -7313,11 +7317,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>3Q25 take rate</t>
-        </is>
-      </c>
-      <c r="B54" s="11">
-        <f>F23/100</f>
+          <t>3Q25 revenue ($M)</t>
+        </is>
+      </c>
+      <c r="B54" s="15">
+        <f>E23</f>
         <v/>
       </c>
       <c r="C54" s="2" t="inlineStr"/>
@@ -7325,26 +7329,23 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>3Q25 North America share of nights</t>
-        </is>
-      </c>
-      <c r="B55" s="10" t="n">
-        <v>0.307</v>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>WS10 10_regional_panel_quarterly.csv, normalised to 100%</t>
-        </is>
-      </c>
+          <t>3Q25 take rate</t>
+        </is>
+      </c>
+      <c r="B55" s="11">
+        <f>F23/100</f>
+        <v/>
+      </c>
+      <c r="C55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>3Q25 EMEA share of nights</t>
+          <t>3Q25 North America share of nights</t>
         </is>
       </c>
       <c r="B56" s="10" t="n">
-        <v>0.4</v>
+        <v>0.307</v>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
@@ -7355,11 +7356,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>3Q25 Latin America share of nights</t>
+          <t>3Q25 EMEA share of nights</t>
         </is>
       </c>
       <c r="B57" s="10" t="n">
-        <v>0.135</v>
+        <v>0.4</v>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
@@ -7370,11 +7371,11 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>3Q25 Asia Pacific share of nights</t>
+          <t>3Q25 Latin America share of nights</t>
         </is>
       </c>
       <c r="B58" s="10" t="n">
-        <v>0.158</v>
+        <v>0.135</v>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
@@ -7385,23 +7386,26 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>4Q25 nights (M)</t>
-        </is>
-      </c>
-      <c r="B59" s="15">
-        <f>B24</f>
-        <v/>
-      </c>
-      <c r="C59" s="2" t="inlineStr"/>
+          <t>3Q25 Asia Pacific share of nights</t>
+        </is>
+      </c>
+      <c r="B59" s="10" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>WS10 10_regional_panel_quarterly.csv, normalised to 100%</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>4Q25 GBV ($M)</t>
+          <t>4Q25 nights (M)</t>
         </is>
       </c>
       <c r="B60" s="15">
-        <f>C24</f>
+        <f>B24</f>
         <v/>
       </c>
       <c r="C60" s="2" t="inlineStr"/>
@@ -7409,11 +7413,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>4Q25 ADR ($)</t>
-        </is>
-      </c>
-      <c r="B61" s="9">
-        <f>D24</f>
+          <t>4Q25 GBV ($M)</t>
+        </is>
+      </c>
+      <c r="B61" s="15">
+        <f>C24</f>
         <v/>
       </c>
       <c r="C61" s="2" t="inlineStr"/>
@@ -7421,11 +7425,11 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>4Q25 revenue ($M)</t>
-        </is>
-      </c>
-      <c r="B62" s="15">
-        <f>E24</f>
+          <t>4Q25 ADR ($)</t>
+        </is>
+      </c>
+      <c r="B62" s="9">
+        <f>D24</f>
         <v/>
       </c>
       <c r="C62" s="2" t="inlineStr"/>
@@ -7433,11 +7437,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>4Q25 take rate</t>
-        </is>
-      </c>
-      <c r="B63" s="11">
-        <f>F24/100</f>
+          <t>4Q25 revenue ($M)</t>
+        </is>
+      </c>
+      <c r="B63" s="15">
+        <f>E24</f>
         <v/>
       </c>
       <c r="C63" s="2" t="inlineStr"/>
@@ -7445,26 +7449,23 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>4Q25 North America share of nights</t>
-        </is>
-      </c>
-      <c r="B64" s="10" t="n">
-        <v>0.2997002997002997</v>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>WS10 10_regional_panel_quarterly.csv, normalised to 100%</t>
-        </is>
-      </c>
+          <t>4Q25 take rate</t>
+        </is>
+      </c>
+      <c r="B64" s="11">
+        <f>F24/100</f>
+        <v/>
+      </c>
+      <c r="C64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>4Q25 EMEA share of nights</t>
+          <t>4Q25 North America share of nights</t>
         </is>
       </c>
       <c r="B65" s="10" t="n">
-        <v>0.3996003996003996</v>
+        <v>0.2997002997002997</v>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
@@ -7475,11 +7476,11 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>4Q25 Latin America share of nights</t>
+          <t>4Q25 EMEA share of nights</t>
         </is>
       </c>
       <c r="B66" s="10" t="n">
-        <v>0.1398601398601399</v>
+        <v>0.3996003996003996</v>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
@@ -7490,11 +7491,11 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>4Q25 Asia Pacific share of nights</t>
+          <t>4Q25 Latin America share of nights</t>
         </is>
       </c>
       <c r="B67" s="10" t="n">
-        <v>0.1608391608391609</v>
+        <v>0.1398601398601399</v>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
@@ -7505,23 +7506,26 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>1Q26 nights (M)</t>
-        </is>
-      </c>
-      <c r="B68" s="15">
-        <f>B25</f>
-        <v/>
-      </c>
-      <c r="C68" s="2" t="inlineStr"/>
+          <t>4Q25 Asia Pacific share of nights</t>
+        </is>
+      </c>
+      <c r="B68" s="10" t="n">
+        <v>0.1608391608391609</v>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>WS10 10_regional_panel_quarterly.csv, normalised to 100%</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1Q26 GBV ($M)</t>
+          <t>1Q26 nights (M)</t>
         </is>
       </c>
       <c r="B69" s="15">
-        <f>C25</f>
+        <f>B25</f>
         <v/>
       </c>
       <c r="C69" s="2" t="inlineStr"/>
@@ -7529,11 +7533,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>1Q26 ADR ($)</t>
-        </is>
-      </c>
-      <c r="B70" s="9">
-        <f>D25</f>
+          <t>1Q26 GBV ($M)</t>
+        </is>
+      </c>
+      <c r="B70" s="15">
+        <f>C25</f>
         <v/>
       </c>
       <c r="C70" s="2" t="inlineStr"/>
@@ -7541,11 +7545,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>1Q26 revenue ($M)</t>
-        </is>
-      </c>
-      <c r="B71" s="15">
-        <f>E25</f>
+          <t>1Q26 ADR ($)</t>
+        </is>
+      </c>
+      <c r="B71" s="9">
+        <f>D25</f>
         <v/>
       </c>
       <c r="C71" s="2" t="inlineStr"/>
@@ -7553,11 +7557,11 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>1Q26 take rate</t>
-        </is>
-      </c>
-      <c r="B72" s="11">
-        <f>F25/100</f>
+          <t>1Q26 revenue ($M)</t>
+        </is>
+      </c>
+      <c r="B72" s="15">
+        <f>E25</f>
         <v/>
       </c>
       <c r="C72" s="2" t="inlineStr"/>
@@ -7565,26 +7569,23 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>1Q26 North America share of nights</t>
-        </is>
-      </c>
-      <c r="B73" s="10" t="n">
-        <v>0.293</v>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>WS10 10_regional_panel_quarterly.csv, normalised to 100%</t>
-        </is>
-      </c>
+          <t>1Q26 take rate</t>
+        </is>
+      </c>
+      <c r="B73" s="11">
+        <f>F25/100</f>
+        <v/>
+      </c>
+      <c r="C73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>1Q26 EMEA share of nights</t>
+          <t>1Q26 North America share of nights</t>
         </is>
       </c>
       <c r="B74" s="10" t="n">
-        <v>0.397</v>
+        <v>0.293</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
@@ -7595,11 +7596,11 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>1Q26 Latin America share of nights</t>
+          <t>1Q26 EMEA share of nights</t>
         </is>
       </c>
       <c r="B75" s="10" t="n">
-        <v>0.147</v>
+        <v>0.397</v>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
@@ -7610,11 +7611,11 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>1Q26 Asia Pacific share of nights</t>
+          <t>1Q26 Latin America share of nights</t>
         </is>
       </c>
       <c r="B76" s="10" t="n">
-        <v>0.163</v>
+        <v>0.147</v>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
@@ -7625,23 +7626,26 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2Q26 nights (M)</t>
-        </is>
-      </c>
-      <c r="B77" s="15">
-        <f>B26</f>
-        <v/>
-      </c>
-      <c r="C77" s="2" t="inlineStr"/>
+          <t>1Q26 Asia Pacific share of nights</t>
+        </is>
+      </c>
+      <c r="B77" s="10" t="n">
+        <v>0.163</v>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>WS10 10_regional_panel_quarterly.csv, normalised to 100%</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2Q26 GBV ($M)</t>
+          <t>2Q26 nights (M)</t>
         </is>
       </c>
       <c r="B78" s="15">
-        <f>C26</f>
+        <f>B26</f>
         <v/>
       </c>
       <c r="C78" s="2" t="inlineStr"/>
@@ -7649,11 +7653,11 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2Q26 ADR ($)</t>
-        </is>
-      </c>
-      <c r="B79" s="9">
-        <f>D26</f>
+          <t>2Q26 GBV ($M)</t>
+        </is>
+      </c>
+      <c r="B79" s="15">
+        <f>C26</f>
         <v/>
       </c>
       <c r="C79" s="2" t="inlineStr"/>
@@ -7661,11 +7665,11 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2Q26 revenue ($M)</t>
-        </is>
-      </c>
-      <c r="B80" s="15">
-        <f>E26</f>
+          <t>2Q26 ADR ($)</t>
+        </is>
+      </c>
+      <c r="B80" s="9">
+        <f>D26</f>
         <v/>
       </c>
       <c r="C80" s="2" t="inlineStr"/>
@@ -7673,11 +7677,11 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2Q26 take rate</t>
-        </is>
-      </c>
-      <c r="B81" s="11">
-        <f>F26/100</f>
+          <t>2Q26 revenue ($M)</t>
+        </is>
+      </c>
+      <c r="B81" s="15">
+        <f>E26</f>
         <v/>
       </c>
       <c r="C81" s="2" t="inlineStr"/>
@@ -7685,26 +7689,23 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2Q26 North America share of nights</t>
-        </is>
-      </c>
-      <c r="B82" s="10" t="n">
-        <v>0.2932932932932933</v>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>WS10 10_regional_panel_quarterly.csv, normalised to 100%</t>
-        </is>
-      </c>
+          <t>2Q26 take rate</t>
+        </is>
+      </c>
+      <c r="B82" s="11">
+        <f>F26/100</f>
+        <v/>
+      </c>
+      <c r="C82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2Q26 EMEA share of nights</t>
+          <t>2Q26 North America share of nights</t>
         </is>
       </c>
       <c r="B83" s="10" t="n">
-        <v>0.3963963963963964</v>
+        <v>0.2932932932932933</v>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
@@ -7715,11 +7716,11 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2Q26 Latin America share of nights</t>
+          <t>2Q26 EMEA share of nights</t>
         </is>
       </c>
       <c r="B84" s="10" t="n">
-        <v>0.1481481481481481</v>
+        <v>0.3963963963963964</v>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
@@ -7730,11 +7731,11 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2Q26 Asia Pacific share of nights</t>
+          <t>2Q26 Latin America share of nights</t>
         </is>
       </c>
       <c r="B85" s="10" t="n">
-        <v>0.1621621621621621</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
@@ -7745,26 +7746,26 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>FY2025 North America share of nights</t>
+          <t>2Q26 Asia Pacific share of nights</t>
         </is>
       </c>
       <c r="B86" s="10" t="n">
-        <v>0.3112886198229538</v>
+        <v>0.1621621621621621</v>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>nights-weighted mean of the four 2025 quarters (WS10)</t>
+          <t>WS10 10_regional_panel_quarterly.csv, normalised to 100%</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>FY2025 EMEA share of nights</t>
+          <t>FY2025 North America share of nights</t>
         </is>
       </c>
       <c r="B87" s="10" t="n">
-        <v>0.3948337306220984</v>
+        <v>0.3112886198229538</v>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
@@ -7775,11 +7776,11 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>FY2025 Latin America share of nights</t>
+          <t>FY2025 EMEA share of nights</t>
         </is>
       </c>
       <c r="B88" s="10" t="n">
-        <v>0.1358071197095587</v>
+        <v>0.3948337306220984</v>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
@@ -7790,11 +7791,11 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>FY2025 Asia Pacific share of nights</t>
+          <t>FY2025 Latin America share of nights</t>
         </is>
       </c>
       <c r="B89" s="10" t="n">
-        <v>0.1580705298453891</v>
+        <v>0.1358071197095587</v>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
@@ -7805,26 +7806,26 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Memo: seasonal adj. EBITDA margin spread, 1Q, 2023-2025 mean (pts vs the full year)</t>
+          <t>FY2025 Asia Pacific share of nights</t>
         </is>
       </c>
       <c r="B90" s="10" t="n">
-        <v>-0.1857930829959057</v>
+        <v>0.1580705298453891</v>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>not used by any formula: the 2027 quarterly margins run off the 2026 spread instead, so 3Q27 stays continuous with the 3Q26 card margin</t>
+          <t>nights-weighted mean of the four 2025 quarters (WS10)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Memo: seasonal adj. EBITDA margin spread, 2Q, 2023-2025 mean (pts vs the full year)</t>
+          <t>Memo: seasonal adj. EBITDA margin spread, 1Q, 2023-2025 mean (pts vs the full year)</t>
         </is>
       </c>
       <c r="B91" s="10" t="n">
-        <v>-0.03045974966257241</v>
+        <v>-0.1857930829959057</v>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
@@ -7835,11 +7836,11 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Memo: seasonal adj. EBITDA margin spread, 3Q, 2023-2025 mean (pts vs the full year)</t>
+          <t>Memo: seasonal adj. EBITDA margin spread, 2Q, 2023-2025 mean (pts vs the full year)</t>
         </is>
       </c>
       <c r="B92" s="10" t="n">
-        <v>0.1608735836707609</v>
+        <v>-0.03045974966257241</v>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
@@ -7850,11 +7851,11 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Memo: seasonal adj. EBITDA margin spread, 4Q, 2023-2025 mean (pts vs the full year)</t>
+          <t>Memo: seasonal adj. EBITDA margin spread, 3Q, 2023-2025 mean (pts vs the full year)</t>
         </is>
       </c>
       <c r="B93" s="10" t="n">
-        <v>-0.05312641632923909</v>
+        <v>0.1608735836707609</v>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
@@ -7865,87 +7866,86 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Seasonal share of full-year nights / revenue, 1Q</t>
+          <t>Memo: seasonal adj. EBITDA margin spread, 4Q, 2023-2025 mean (pts vs the full year)</t>
         </is>
       </c>
       <c r="B94" s="10" t="n">
-        <v>0.269486182357886</v>
+        <v>-0.05312641632923909</v>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>2023-2025 mean; revenue share 18.7%</t>
+          <t>not used by any formula: the 2027 quarterly margins run off the 2026 spread instead, so 3Q27 stays continuous with the 3Q26 card margin</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Seasonal share of full-year nights / revenue, 2Q</t>
+          <t>Seasonal share of full-year nights / revenue, 1Q</t>
         </is>
       </c>
       <c r="B95" s="10" t="n">
-        <v>0.254496518186287</v>
+        <v>0.269486182357886</v>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>2023-2025 mean; revenue share 25.0%</t>
+          <t>2023-2025 mean; revenue share 18.7%</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Seasonal share of full-year nights / revenue, 3Q</t>
+          <t>Seasonal share of full-year nights / revenue, 2Q</t>
         </is>
       </c>
       <c r="B96" s="10" t="n">
-        <v>0.2510232950479808</v>
+        <v>0.254496518186287</v>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>2023-2025 mean; revenue share 33.8%</t>
+          <t>2023-2025 mean; revenue share 25.0%</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Seasonal share of full-year nights / revenue, 4Q</t>
+          <t>Seasonal share of full-year nights / revenue, 3Q</t>
         </is>
       </c>
       <c r="B97" s="10" t="n">
-        <v>0.2249940044078461</v>
+        <v>0.2510232950479808</v>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>2023-2025 mean; revenue share 22.5%</t>
+          <t>2023-2025 mean; revenue share 33.8%</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>1Q26 adj. EBITDA margin (actual)</t>
-        </is>
-      </c>
-      <c r="B98" s="11">
-        <f>H25/100</f>
-        <v/>
+          <t>Seasonal share of full-year nights / revenue, 4Q</t>
+        </is>
+      </c>
+      <c r="B98" s="10" t="n">
+        <v>0.2249940044078461</v>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>actual; used as the 2027 seasonal template</t>
+          <t>2023-2025 mean; revenue share 22.5%</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2Q26 adj. EBITDA margin (actual)</t>
+          <t>1Q26 adj. EBITDA margin (actual)</t>
         </is>
       </c>
       <c r="B99" s="11">
-        <f>H26/100</f>
+        <f>H25/100</f>
         <v/>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -7957,26 +7957,27 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>LTM revenue ($M)</t>
-        </is>
-      </c>
-      <c r="B100" s="15" t="n">
-        <v>13159</v>
+          <t>2Q26 adj. EBITDA margin (actual)</t>
+        </is>
+      </c>
+      <c r="B100" s="11">
+        <f>H26/100</f>
+        <v/>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>3Q25-2Q26</t>
+          <t>actual; used as the 2027 seasonal template</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>LTM adj. EBITDA ($M)</t>
-        </is>
-      </c>
-      <c r="B101" s="15" t="n">
-        <v>4617</v>
+          <t>LTM revenue ($M)</t>
+        </is>
+      </c>
+      <c r="B101" s="14" t="n">
+        <v>13159</v>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
@@ -7987,11 +7988,11 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>LTM FCF ($M)</t>
-        </is>
-      </c>
-      <c r="B102" s="15" t="n">
-        <v>4827</v>
+          <t>LTM adj. EBITDA ($M)</t>
+        </is>
+      </c>
+      <c r="B102" s="14" t="n">
+        <v>4617</v>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
@@ -8002,15 +8003,228 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
+          <t>LTM FCF ($M)</t>
+        </is>
+      </c>
+      <c r="B103" s="14" t="n">
+        <v>4827</v>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>3Q25-2Q26</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
           <t>LTM SBC ($M)</t>
         </is>
       </c>
-      <c r="B103" s="15" t="n">
+      <c r="B104" s="14" t="n">
         <v>1696</v>
       </c>
-      <c r="C103" s="2" t="inlineStr">
+      <c r="C104" s="2" t="inlineStr">
         <is>
           <t>3Q25-2Q26</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
+        <is>
+          <t>FY2025 CASH-BRIDGE ANCHORS - the FY2025A memo column on Costs and Cash. No forecast year depends on these.</t>
+        </is>
+      </c>
+      <c r="B106" s="6" t="n"/>
+      <c r="C106" s="6" t="n"/>
+      <c r="D106" s="6" t="n"/>
+      <c r="E106" s="6" t="n"/>
+      <c r="F106" s="6" t="n"/>
+      <c r="G106" s="6" t="n"/>
+      <c r="H106" s="6" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C107" s="7" t="inlineStr">
+        <is>
+          <t>Source / formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>FY2025 D&amp;A ($M)</t>
+        </is>
+      </c>
+      <c r="B108" s="14" t="n">
+        <v>91</v>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>data/processed/abnb_fcf_bridge.csv, sum of 1Q25-4Q25 (da)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>FY2025 D&amp;A and other add-backs ($M)</t>
+        </is>
+      </c>
+      <c r="B109" s="14" t="n">
+        <v>161</v>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>data/processed/abnb_fcf_bridge.csv, sum of 1Q25-4Q25 (da 91 + other_addbacks 70)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>FY2025 interest income ($M)</t>
+        </is>
+      </c>
+      <c r="B110" s="14" t="n">
+        <v>705</v>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>data/processed/abnb_fcf_bridge.csv, sum of 1Q25-4Q25 (interest_income)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>FY2025 interest expense ($M)</t>
+        </is>
+      </c>
+      <c r="B111" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>data/processed/abnb_fcf_bridge.csv, sum of 1Q25-4Q25 reports zero in every quarter of 2025; the note coupon sits inside other income/(expense) in that bridge. Memo only - the forecast years take interest expense from Inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>FY2025 other income / (expense) ($M)</t>
+        </is>
+      </c>
+      <c r="B112" s="14" t="n">
+        <v>-112</v>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>data/processed/abnb_fcf_bridge.csv, sum of 1Q25-4Q25 (other_income_expense)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>FY2025 cash taxes ($M)</t>
+        </is>
+      </c>
+      <c r="B113" s="14" t="n">
+        <v>-232</v>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>WS07: FY2025 cash taxes 1.9% of revenue (0.019 x $12,241M = $232M); the book tax provision was $626M</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>FY2025 change in unearned fees ($M)</t>
+        </is>
+      </c>
+      <c r="B114" s="14" t="n">
+        <v>127</v>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>data/processed/abnb_fcf_bridge.csv, sum of 1Q25-4Q25 (change_unearned_fees)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>FY2025 working-capital residual ($M)</t>
+        </is>
+      </c>
+      <c r="B115" s="14" t="n">
+        <v>-139</v>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>WS07: FY24 and FY25 both about -$140M. With the eight lines above this reproduces the reported FY2025 FCF of $4,613M exactly</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>FY2025 capex ($M)</t>
+        </is>
+      </c>
+      <c r="B116" s="14" t="n">
+        <v>-33</v>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>data/processed/abnb_fcf_bridge.csv, sum of 1Q25-4Q25 (capex)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>FY2025 buybacks ($M)</t>
+        </is>
+      </c>
+      <c r="B117" s="15">
+        <f>K21+K22+K23+K24</f>
+        <v/>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>sum of the 2025 quarters above</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>FY2025 RSU tax withholding ($M)</t>
+        </is>
+      </c>
+      <c r="B118" s="15">
+        <f>L21+L22+L23+L24</f>
+        <v/>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>sum of the 2025 quarters above</t>
         </is>
       </c>
     </row>
@@ -8143,19 +8357,19 @@
         </is>
       </c>
       <c r="C6" s="15">
-        <f>History!$B$50*History!$B$55</f>
+        <f>History!$B$51*History!$B$56</f>
         <v/>
       </c>
       <c r="D6" s="15">
-        <f>History!$B$59*History!$B$64</f>
+        <f>History!$B$60*History!$B$65</f>
         <v/>
       </c>
       <c r="E6" s="15">
-        <f>History!$B$68*History!$B$73</f>
+        <f>History!$B$69*History!$B$74</f>
         <v/>
       </c>
       <c r="F6" s="15">
-        <f>History!$B$77*History!$B$82</f>
+        <f>History!$B$78*History!$B$83</f>
         <v/>
       </c>
       <c r="G6" s="15">
@@ -8179,19 +8393,19 @@
         </is>
       </c>
       <c r="C7" s="15">
-        <f>History!$B$50*History!$B$56</f>
+        <f>History!$B$51*History!$B$57</f>
         <v/>
       </c>
       <c r="D7" s="15">
-        <f>History!$B$59*History!$B$65</f>
+        <f>History!$B$60*History!$B$66</f>
         <v/>
       </c>
       <c r="E7" s="15">
-        <f>History!$B$68*History!$B$74</f>
+        <f>History!$B$69*History!$B$75</f>
         <v/>
       </c>
       <c r="F7" s="15">
-        <f>History!$B$77*History!$B$83</f>
+        <f>History!$B$78*History!$B$84</f>
         <v/>
       </c>
       <c r="G7" s="15">
@@ -8215,19 +8429,19 @@
         </is>
       </c>
       <c r="C8" s="15">
-        <f>History!$B$50*History!$B$57</f>
+        <f>History!$B$51*History!$B$58</f>
         <v/>
       </c>
       <c r="D8" s="15">
-        <f>History!$B$59*History!$B$66</f>
+        <f>History!$B$60*History!$B$67</f>
         <v/>
       </c>
       <c r="E8" s="15">
-        <f>History!$B$68*History!$B$75</f>
+        <f>History!$B$69*History!$B$76</f>
         <v/>
       </c>
       <c r="F8" s="15">
-        <f>History!$B$77*History!$B$84</f>
+        <f>History!$B$78*History!$B$85</f>
         <v/>
       </c>
       <c r="G8" s="15">
@@ -8251,19 +8465,19 @@
         </is>
       </c>
       <c r="C9" s="15">
-        <f>History!$B$50*History!$B$58</f>
+        <f>History!$B$51*History!$B$59</f>
         <v/>
       </c>
       <c r="D9" s="15">
-        <f>History!$B$59*History!$B$67</f>
+        <f>History!$B$60*History!$B$68</f>
         <v/>
       </c>
       <c r="E9" s="15">
-        <f>History!$B$68*History!$B$76</f>
+        <f>History!$B$69*History!$B$77</f>
         <v/>
       </c>
       <c r="F9" s="15">
-        <f>History!$B$77*History!$B$85</f>
+        <f>History!$B$78*History!$B$86</f>
         <v/>
       </c>
       <c r="G9" s="15">
@@ -8831,19 +9045,19 @@
         </is>
       </c>
       <c r="C23" s="20">
-        <f>C22/History!$B$50-1</f>
+        <f>C22/History!$B$51-1</f>
         <v/>
       </c>
       <c r="D23" s="20">
-        <f>D22/History!$B$59-1</f>
+        <f>D22/History!$B$60-1</f>
         <v/>
       </c>
       <c r="E23" s="20">
-        <f>E22/History!$B$68-1</f>
+        <f>E22/History!$B$69-1</f>
         <v/>
       </c>
       <c r="F23" s="20">
-        <f>F22/History!$B$77-1</f>
+        <f>F22/History!$B$78-1</f>
         <v/>
       </c>
       <c r="G23" s="20">
@@ -8959,19 +9173,19 @@
         </is>
       </c>
       <c r="C26" s="9">
-        <f>History!$B$52*(1+C24)*(1+C25)</f>
+        <f>History!$B$53*(1+C24)*(1+C25)</f>
         <v/>
       </c>
       <c r="D26" s="9">
-        <f>History!$B$61*(1+D24)*(1+D25)</f>
+        <f>History!$B$62*(1+D24)*(1+D25)</f>
         <v/>
       </c>
       <c r="E26" s="9">
-        <f>History!$B$70*(1+E24)*(1+E25)</f>
+        <f>History!$B$71*(1+E24)*(1+E25)</f>
         <v/>
       </c>
       <c r="F26" s="9">
-        <f>History!$B$79*(1+F24)*(1+F25)</f>
+        <f>History!$B$80*(1+F24)*(1+F25)</f>
         <v/>
       </c>
       <c r="G26" s="9">
@@ -9007,19 +9221,19 @@
         </is>
       </c>
       <c r="C27" s="20">
-        <f>C26/History!$B$52-1</f>
+        <f>C26/History!$B$53-1</f>
         <v/>
       </c>
       <c r="D27" s="20">
-        <f>D26/History!$B$61-1</f>
+        <f>D26/History!$B$62-1</f>
         <v/>
       </c>
       <c r="E27" s="20">
-        <f>E26/History!$B$70-1</f>
+        <f>E26/History!$B$71-1</f>
         <v/>
       </c>
       <c r="F27" s="20">
-        <f>F26/History!$B$79-1</f>
+        <f>F26/History!$B$80-1</f>
         <v/>
       </c>
       <c r="G27" s="20">
@@ -9103,19 +9317,19 @@
         </is>
       </c>
       <c r="C29" s="20">
-        <f>C28/History!$B$51-1</f>
+        <f>C28/History!$B$52-1</f>
         <v/>
       </c>
       <c r="D29" s="20">
-        <f>D28/History!$B$60-1</f>
+        <f>D28/History!$B$61-1</f>
         <v/>
       </c>
       <c r="E29" s="20">
-        <f>E28/History!$B$69-1</f>
+        <f>E28/History!$B$70-1</f>
         <v/>
       </c>
       <c r="F29" s="20">
-        <f>F28/History!$B$78-1</f>
+        <f>F28/History!$B$79-1</f>
         <v/>
       </c>
       <c r="G29" s="20">
@@ -9151,19 +9365,19 @@
         </is>
       </c>
       <c r="C30" s="11">
-        <f>History!$B$54+Inputs!$C$26/10000</f>
+        <f>History!$B$55+Inputs!$C$26/10000</f>
         <v/>
       </c>
       <c r="D30" s="11">
-        <f>History!$B$63+Inputs!$C$26/10000</f>
+        <f>History!$B$64+Inputs!$C$26/10000</f>
         <v/>
       </c>
       <c r="E30" s="11">
-        <f>History!$B$72+Inputs!$C$49/10000</f>
+        <f>History!$B$73+Inputs!$C$49/10000</f>
         <v/>
       </c>
       <c r="F30" s="11">
-        <f>History!$B$81+Inputs!$C$49/10000</f>
+        <f>History!$B$82+Inputs!$C$49/10000</f>
         <v/>
       </c>
       <c r="G30" s="11">
@@ -9311,7 +9525,7 @@
         <v/>
       </c>
       <c r="K33" s="21">
-        <f>K28*(J30+Inputs!$C$72/10000)*(1+K32)</f>
+        <f>K28*K30*(1+K32)</f>
         <v/>
       </c>
     </row>
@@ -9471,19 +9685,19 @@
         </is>
       </c>
       <c r="C37" s="23">
-        <f>C36/History!$B$53-1</f>
+        <f>C36/History!$B$54-1</f>
         <v/>
       </c>
       <c r="D37" s="23">
-        <f>D36/History!$B$62-1</f>
+        <f>D36/History!$B$63-1</f>
         <v/>
       </c>
       <c r="E37" s="23">
-        <f>E36/History!$B$71-1</f>
+        <f>E36/History!$B$72-1</f>
         <v/>
       </c>
       <c r="F37" s="23">
-        <f>F36/History!$B$80-1</f>
+        <f>F36/History!$B$81-1</f>
         <v/>
       </c>
       <c r="G37" s="23">
@@ -9519,11 +9733,11 @@
         </is>
       </c>
       <c r="E38" s="11">
-        <f>History!$B$98-Costs!$D$22</f>
+        <f>History!$B$99-Costs!$D$22</f>
         <v/>
       </c>
       <c r="F38" s="11">
-        <f>History!$B$99-Costs!$D$22</f>
+        <f>History!$B$100-Costs!$D$22</f>
         <v/>
       </c>
       <c r="G38" s="11">
@@ -9707,27 +9921,27 @@
         </is>
       </c>
       <c r="C43" s="20">
+        <f>History!$B$97</f>
+        <v/>
+      </c>
+      <c r="D43" s="20">
+        <f>History!$B$98</f>
+        <v/>
+      </c>
+      <c r="E43" s="20">
+        <f>History!$B$95</f>
+        <v/>
+      </c>
+      <c r="F43" s="20">
         <f>History!$B$96</f>
         <v/>
       </c>
-      <c r="D43" s="20">
+      <c r="G43" s="20">
         <f>History!$B$97</f>
         <v/>
       </c>
-      <c r="E43" s="20">
-        <f>History!$B$94</f>
-        <v/>
-      </c>
-      <c r="F43" s="20">
-        <f>History!$B$95</f>
-        <v/>
-      </c>
-      <c r="G43" s="20">
-        <f>History!$B$96</f>
-        <v/>
-      </c>
       <c r="H43" s="20">
-        <f>History!$B$97</f>
+        <f>History!$B$98</f>
         <v/>
       </c>
     </row>
@@ -9818,19 +10032,19 @@
         </is>
       </c>
       <c r="C47" s="15">
-        <f>History!$B$50*History!$B$55</f>
+        <f>History!$B$51*History!$B$56</f>
         <v/>
       </c>
       <c r="D47" s="15">
-        <f>History!$B$59*History!$B$64</f>
+        <f>History!$B$60*History!$B$65</f>
         <v/>
       </c>
       <c r="E47" s="15">
-        <f>History!$B$68*History!$B$73</f>
+        <f>History!$B$69*History!$B$74</f>
         <v/>
       </c>
       <c r="F47" s="15">
-        <f>History!$B$77*History!$B$82</f>
+        <f>History!$B$78*History!$B$83</f>
         <v/>
       </c>
       <c r="G47" s="15">
@@ -9854,19 +10068,19 @@
         </is>
       </c>
       <c r="C48" s="15">
-        <f>History!$B$50*History!$B$56</f>
+        <f>History!$B$51*History!$B$57</f>
         <v/>
       </c>
       <c r="D48" s="15">
-        <f>History!$B$59*History!$B$65</f>
+        <f>History!$B$60*History!$B$66</f>
         <v/>
       </c>
       <c r="E48" s="15">
-        <f>History!$B$68*History!$B$74</f>
+        <f>History!$B$69*History!$B$75</f>
         <v/>
       </c>
       <c r="F48" s="15">
-        <f>History!$B$77*History!$B$83</f>
+        <f>History!$B$78*History!$B$84</f>
         <v/>
       </c>
       <c r="G48" s="15">
@@ -9890,19 +10104,19 @@
         </is>
       </c>
       <c r="C49" s="15">
-        <f>History!$B$50*History!$B$57</f>
+        <f>History!$B$51*History!$B$58</f>
         <v/>
       </c>
       <c r="D49" s="15">
-        <f>History!$B$59*History!$B$66</f>
+        <f>History!$B$60*History!$B$67</f>
         <v/>
       </c>
       <c r="E49" s="15">
-        <f>History!$B$68*History!$B$75</f>
+        <f>History!$B$69*History!$B$76</f>
         <v/>
       </c>
       <c r="F49" s="15">
-        <f>History!$B$77*History!$B$84</f>
+        <f>History!$B$78*History!$B$85</f>
         <v/>
       </c>
       <c r="G49" s="15">
@@ -9926,19 +10140,19 @@
         </is>
       </c>
       <c r="C50" s="15">
-        <f>History!$B$50*History!$B$58</f>
+        <f>History!$B$51*History!$B$59</f>
         <v/>
       </c>
       <c r="D50" s="15">
-        <f>History!$B$59*History!$B$67</f>
+        <f>History!$B$60*History!$B$68</f>
         <v/>
       </c>
       <c r="E50" s="15">
-        <f>History!$B$68*History!$B$76</f>
+        <f>History!$B$69*History!$B$77</f>
         <v/>
       </c>
       <c r="F50" s="15">
-        <f>History!$B$77*History!$B$85</f>
+        <f>History!$B$78*History!$B$86</f>
         <v/>
       </c>
       <c r="G50" s="15">
@@ -10506,19 +10720,19 @@
         </is>
       </c>
       <c r="C64" s="20">
-        <f>C63/History!$B$50-1</f>
+        <f>C63/History!$B$51-1</f>
         <v/>
       </c>
       <c r="D64" s="20">
-        <f>D63/History!$B$59-1</f>
+        <f>D63/History!$B$60-1</f>
         <v/>
       </c>
       <c r="E64" s="20">
-        <f>E63/History!$B$68-1</f>
+        <f>E63/History!$B$69-1</f>
         <v/>
       </c>
       <c r="F64" s="20">
-        <f>F63/History!$B$77-1</f>
+        <f>F63/History!$B$78-1</f>
         <v/>
       </c>
       <c r="G64" s="20">
@@ -10634,19 +10848,19 @@
         </is>
       </c>
       <c r="C67" s="9">
-        <f>History!$B$52*(1+C65)*(1+C66)</f>
+        <f>History!$B$53*(1+C65)*(1+C66)</f>
         <v/>
       </c>
       <c r="D67" s="9">
-        <f>History!$B$61*(1+D65)*(1+D66)</f>
+        <f>History!$B$62*(1+D65)*(1+D66)</f>
         <v/>
       </c>
       <c r="E67" s="9">
-        <f>History!$B$70*(1+E65)*(1+E66)</f>
+        <f>History!$B$71*(1+E65)*(1+E66)</f>
         <v/>
       </c>
       <c r="F67" s="9">
-        <f>History!$B$79*(1+F65)*(1+F66)</f>
+        <f>History!$B$80*(1+F65)*(1+F66)</f>
         <v/>
       </c>
       <c r="G67" s="9">
@@ -10682,19 +10896,19 @@
         </is>
       </c>
       <c r="C68" s="20">
-        <f>C67/History!$B$52-1</f>
+        <f>C67/History!$B$53-1</f>
         <v/>
       </c>
       <c r="D68" s="20">
-        <f>D67/History!$B$61-1</f>
+        <f>D67/History!$B$62-1</f>
         <v/>
       </c>
       <c r="E68" s="20">
-        <f>E67/History!$B$70-1</f>
+        <f>E67/History!$B$71-1</f>
         <v/>
       </c>
       <c r="F68" s="20">
-        <f>F67/History!$B$79-1</f>
+        <f>F67/History!$B$80-1</f>
         <v/>
       </c>
       <c r="G68" s="20">
@@ -10778,19 +10992,19 @@
         </is>
       </c>
       <c r="C70" s="20">
-        <f>C69/History!$B$51-1</f>
+        <f>C69/History!$B$52-1</f>
         <v/>
       </c>
       <c r="D70" s="20">
-        <f>D69/History!$B$60-1</f>
+        <f>D69/History!$B$61-1</f>
         <v/>
       </c>
       <c r="E70" s="20">
-        <f>E69/History!$B$69-1</f>
+        <f>E69/History!$B$70-1</f>
         <v/>
       </c>
       <c r="F70" s="20">
-        <f>F69/History!$B$78-1</f>
+        <f>F69/History!$B$79-1</f>
         <v/>
       </c>
       <c r="G70" s="20">
@@ -10826,19 +11040,19 @@
         </is>
       </c>
       <c r="C71" s="11">
-        <f>History!$B$54+Inputs!$D$26/10000</f>
+        <f>History!$B$55+Inputs!$D$26/10000</f>
         <v/>
       </c>
       <c r="D71" s="11">
-        <f>History!$B$63+Inputs!$D$26/10000</f>
+        <f>History!$B$64+Inputs!$D$26/10000</f>
         <v/>
       </c>
       <c r="E71" s="11">
-        <f>History!$B$72+Inputs!$D$49/10000</f>
+        <f>History!$B$73+Inputs!$D$49/10000</f>
         <v/>
       </c>
       <c r="F71" s="11">
-        <f>History!$B$81+Inputs!$D$49/10000</f>
+        <f>History!$B$82+Inputs!$D$49/10000</f>
         <v/>
       </c>
       <c r="G71" s="11">
@@ -10986,7 +11200,7 @@
         <v/>
       </c>
       <c r="K74" s="21">
-        <f>K69*(J71+Inputs!$D$72/10000)*(1+K73)</f>
+        <f>K69*K71*(1+K73)</f>
         <v/>
       </c>
     </row>
@@ -11146,19 +11360,19 @@
         </is>
       </c>
       <c r="C78" s="23">
-        <f>C77/History!$B$53-1</f>
+        <f>C77/History!$B$54-1</f>
         <v/>
       </c>
       <c r="D78" s="23">
-        <f>D77/History!$B$62-1</f>
+        <f>D77/History!$B$63-1</f>
         <v/>
       </c>
       <c r="E78" s="23">
-        <f>E77/History!$B$71-1</f>
+        <f>E77/History!$B$72-1</f>
         <v/>
       </c>
       <c r="F78" s="23">
-        <f>F77/History!$B$80-1</f>
+        <f>F77/History!$B$81-1</f>
         <v/>
       </c>
       <c r="G78" s="23">
@@ -11194,11 +11408,11 @@
         </is>
       </c>
       <c r="E79" s="11">
-        <f>History!$B$98-Costs!$D$52</f>
+        <f>History!$B$99-Costs!$D$52</f>
         <v/>
       </c>
       <c r="F79" s="11">
-        <f>History!$B$99-Costs!$D$52</f>
+        <f>History!$B$100-Costs!$D$52</f>
         <v/>
       </c>
       <c r="G79" s="11">
@@ -11382,27 +11596,27 @@
         </is>
       </c>
       <c r="C84" s="20">
+        <f>History!$B$97</f>
+        <v/>
+      </c>
+      <c r="D84" s="20">
+        <f>History!$B$98</f>
+        <v/>
+      </c>
+      <c r="E84" s="20">
+        <f>History!$B$95</f>
+        <v/>
+      </c>
+      <c r="F84" s="20">
         <f>History!$B$96</f>
         <v/>
       </c>
-      <c r="D84" s="20">
+      <c r="G84" s="20">
         <f>History!$B$97</f>
         <v/>
       </c>
-      <c r="E84" s="20">
-        <f>History!$B$94</f>
-        <v/>
-      </c>
-      <c r="F84" s="20">
-        <f>History!$B$95</f>
-        <v/>
-      </c>
-      <c r="G84" s="20">
-        <f>History!$B$96</f>
-        <v/>
-      </c>
       <c r="H84" s="20">
-        <f>History!$B$97</f>
+        <f>History!$B$98</f>
         <v/>
       </c>
     </row>
@@ -11493,19 +11707,19 @@
         </is>
       </c>
       <c r="C88" s="15">
-        <f>History!$B$50*History!$B$55</f>
+        <f>History!$B$51*History!$B$56</f>
         <v/>
       </c>
       <c r="D88" s="15">
-        <f>History!$B$59*History!$B$64</f>
+        <f>History!$B$60*History!$B$65</f>
         <v/>
       </c>
       <c r="E88" s="15">
-        <f>History!$B$68*History!$B$73</f>
+        <f>History!$B$69*History!$B$74</f>
         <v/>
       </c>
       <c r="F88" s="15">
-        <f>History!$B$77*History!$B$82</f>
+        <f>History!$B$78*History!$B$83</f>
         <v/>
       </c>
       <c r="G88" s="15">
@@ -11529,19 +11743,19 @@
         </is>
       </c>
       <c r="C89" s="15">
-        <f>History!$B$50*History!$B$56</f>
+        <f>History!$B$51*History!$B$57</f>
         <v/>
       </c>
       <c r="D89" s="15">
-        <f>History!$B$59*History!$B$65</f>
+        <f>History!$B$60*History!$B$66</f>
         <v/>
       </c>
       <c r="E89" s="15">
-        <f>History!$B$68*History!$B$74</f>
+        <f>History!$B$69*History!$B$75</f>
         <v/>
       </c>
       <c r="F89" s="15">
-        <f>History!$B$77*History!$B$83</f>
+        <f>History!$B$78*History!$B$84</f>
         <v/>
       </c>
       <c r="G89" s="15">
@@ -11565,19 +11779,19 @@
         </is>
       </c>
       <c r="C90" s="15">
-        <f>History!$B$50*History!$B$57</f>
+        <f>History!$B$51*History!$B$58</f>
         <v/>
       </c>
       <c r="D90" s="15">
-        <f>History!$B$59*History!$B$66</f>
+        <f>History!$B$60*History!$B$67</f>
         <v/>
       </c>
       <c r="E90" s="15">
-        <f>History!$B$68*History!$B$75</f>
+        <f>History!$B$69*History!$B$76</f>
         <v/>
       </c>
       <c r="F90" s="15">
-        <f>History!$B$77*History!$B$84</f>
+        <f>History!$B$78*History!$B$85</f>
         <v/>
       </c>
       <c r="G90" s="15">
@@ -11601,19 +11815,19 @@
         </is>
       </c>
       <c r="C91" s="15">
-        <f>History!$B$50*History!$B$58</f>
+        <f>History!$B$51*History!$B$59</f>
         <v/>
       </c>
       <c r="D91" s="15">
-        <f>History!$B$59*History!$B$67</f>
+        <f>History!$B$60*History!$B$68</f>
         <v/>
       </c>
       <c r="E91" s="15">
-        <f>History!$B$68*History!$B$76</f>
+        <f>History!$B$69*History!$B$77</f>
         <v/>
       </c>
       <c r="F91" s="15">
-        <f>History!$B$77*History!$B$85</f>
+        <f>History!$B$78*History!$B$86</f>
         <v/>
       </c>
       <c r="G91" s="15">
@@ -12181,19 +12395,19 @@
         </is>
       </c>
       <c r="C105" s="20">
-        <f>C104/History!$B$50-1</f>
+        <f>C104/History!$B$51-1</f>
         <v/>
       </c>
       <c r="D105" s="20">
-        <f>D104/History!$B$59-1</f>
+        <f>D104/History!$B$60-1</f>
         <v/>
       </c>
       <c r="E105" s="20">
-        <f>E104/History!$B$68-1</f>
+        <f>E104/History!$B$69-1</f>
         <v/>
       </c>
       <c r="F105" s="20">
-        <f>F104/History!$B$77-1</f>
+        <f>F104/History!$B$78-1</f>
         <v/>
       </c>
       <c r="G105" s="20">
@@ -12309,19 +12523,19 @@
         </is>
       </c>
       <c r="C108" s="9">
-        <f>History!$B$52*(1+C106)*(1+C107)</f>
+        <f>History!$B$53*(1+C106)*(1+C107)</f>
         <v/>
       </c>
       <c r="D108" s="9">
-        <f>History!$B$61*(1+D106)*(1+D107)</f>
+        <f>History!$B$62*(1+D106)*(1+D107)</f>
         <v/>
       </c>
       <c r="E108" s="9">
-        <f>History!$B$70*(1+E106)*(1+E107)</f>
+        <f>History!$B$71*(1+E106)*(1+E107)</f>
         <v/>
       </c>
       <c r="F108" s="9">
-        <f>History!$B$79*(1+F106)*(1+F107)</f>
+        <f>History!$B$80*(1+F106)*(1+F107)</f>
         <v/>
       </c>
       <c r="G108" s="9">
@@ -12357,19 +12571,19 @@
         </is>
       </c>
       <c r="C109" s="20">
-        <f>C108/History!$B$52-1</f>
+        <f>C108/History!$B$53-1</f>
         <v/>
       </c>
       <c r="D109" s="20">
-        <f>D108/History!$B$61-1</f>
+        <f>D108/History!$B$62-1</f>
         <v/>
       </c>
       <c r="E109" s="20">
-        <f>E108/History!$B$70-1</f>
+        <f>E108/History!$B$71-1</f>
         <v/>
       </c>
       <c r="F109" s="20">
-        <f>F108/History!$B$79-1</f>
+        <f>F108/History!$B$80-1</f>
         <v/>
       </c>
       <c r="G109" s="20">
@@ -12453,19 +12667,19 @@
         </is>
       </c>
       <c r="C111" s="20">
-        <f>C110/History!$B$51-1</f>
+        <f>C110/History!$B$52-1</f>
         <v/>
       </c>
       <c r="D111" s="20">
-        <f>D110/History!$B$60-1</f>
+        <f>D110/History!$B$61-1</f>
         <v/>
       </c>
       <c r="E111" s="20">
-        <f>E110/History!$B$69-1</f>
+        <f>E110/History!$B$70-1</f>
         <v/>
       </c>
       <c r="F111" s="20">
-        <f>F110/History!$B$78-1</f>
+        <f>F110/History!$B$79-1</f>
         <v/>
       </c>
       <c r="G111" s="20">
@@ -12501,19 +12715,19 @@
         </is>
       </c>
       <c r="C112" s="11">
-        <f>History!$B$54+Inputs!$E$26/10000</f>
+        <f>History!$B$55+Inputs!$E$26/10000</f>
         <v/>
       </c>
       <c r="D112" s="11">
-        <f>History!$B$63+Inputs!$E$26/10000</f>
+        <f>History!$B$64+Inputs!$E$26/10000</f>
         <v/>
       </c>
       <c r="E112" s="11">
-        <f>History!$B$72+Inputs!$E$49/10000</f>
+        <f>History!$B$73+Inputs!$E$49/10000</f>
         <v/>
       </c>
       <c r="F112" s="11">
-        <f>History!$B$81+Inputs!$E$49/10000</f>
+        <f>History!$B$82+Inputs!$E$49/10000</f>
         <v/>
       </c>
       <c r="G112" s="11">
@@ -12661,7 +12875,7 @@
         <v/>
       </c>
       <c r="K115" s="21">
-        <f>K110*(J112+Inputs!$E$72/10000)*(1+K114)</f>
+        <f>K110*K112*(1+K114)</f>
         <v/>
       </c>
     </row>
@@ -12821,19 +13035,19 @@
         </is>
       </c>
       <c r="C119" s="23">
-        <f>C118/History!$B$53-1</f>
+        <f>C118/History!$B$54-1</f>
         <v/>
       </c>
       <c r="D119" s="23">
-        <f>D118/History!$B$62-1</f>
+        <f>D118/History!$B$63-1</f>
         <v/>
       </c>
       <c r="E119" s="23">
-        <f>E118/History!$B$71-1</f>
+        <f>E118/History!$B$72-1</f>
         <v/>
       </c>
       <c r="F119" s="23">
-        <f>F118/History!$B$80-1</f>
+        <f>F118/History!$B$81-1</f>
         <v/>
       </c>
       <c r="G119" s="23">
@@ -12869,11 +13083,11 @@
         </is>
       </c>
       <c r="E120" s="11">
-        <f>History!$B$98-Costs!$D$82</f>
+        <f>History!$B$99-Costs!$D$82</f>
         <v/>
       </c>
       <c r="F120" s="11">
-        <f>History!$B$99-Costs!$D$82</f>
+        <f>History!$B$100-Costs!$D$82</f>
         <v/>
       </c>
       <c r="G120" s="11">
@@ -13057,27 +13271,27 @@
         </is>
       </c>
       <c r="C125" s="20">
+        <f>History!$B$97</f>
+        <v/>
+      </c>
+      <c r="D125" s="20">
+        <f>History!$B$98</f>
+        <v/>
+      </c>
+      <c r="E125" s="20">
+        <f>History!$B$95</f>
+        <v/>
+      </c>
+      <c r="F125" s="20">
         <f>History!$B$96</f>
         <v/>
       </c>
-      <c r="D125" s="20">
+      <c r="G125" s="20">
         <f>History!$B$97</f>
         <v/>
       </c>
-      <c r="E125" s="20">
-        <f>History!$B$94</f>
-        <v/>
-      </c>
-      <c r="F125" s="20">
-        <f>History!$B$95</f>
-        <v/>
-      </c>
-      <c r="G125" s="20">
-        <f>History!$B$96</f>
-        <v/>
-      </c>
       <c r="H125" s="20">
-        <f>History!$B$97</f>
+        <f>History!$B$98</f>
         <v/>
       </c>
     </row>
@@ -13511,7 +13725,7 @@
         </is>
       </c>
       <c r="C18" s="15">
-        <f>161</f>
+        <f>History!$B$109</f>
         <v/>
       </c>
       <c r="D18" s="15">
@@ -13707,7 +13921,7 @@
         </is>
       </c>
       <c r="C25" s="15">
-        <f>91</f>
+        <f>History!$B$108</f>
         <v/>
       </c>
       <c r="D25" s="15">
@@ -13783,7 +13997,7 @@
         </is>
       </c>
       <c r="C28" s="15">
-        <f>705</f>
+        <f>History!$B$110</f>
         <v/>
       </c>
       <c r="D28" s="15">
@@ -13811,7 +14025,7 @@
         </is>
       </c>
       <c r="C29" s="15">
-        <f>0</f>
+        <f>History!$B$111</f>
         <v/>
       </c>
       <c r="D29" s="15">
@@ -14292,7 +14506,7 @@
         </is>
       </c>
       <c r="C48" s="15">
-        <f>161</f>
+        <f>History!$B$109</f>
         <v/>
       </c>
       <c r="D48" s="15">
@@ -14488,7 +14702,7 @@
         </is>
       </c>
       <c r="C55" s="15">
-        <f>91</f>
+        <f>History!$B$108</f>
         <v/>
       </c>
       <c r="D55" s="15">
@@ -14564,7 +14778,7 @@
         </is>
       </c>
       <c r="C58" s="15">
-        <f>705</f>
+        <f>History!$B$110</f>
         <v/>
       </c>
       <c r="D58" s="15">
@@ -14592,7 +14806,7 @@
         </is>
       </c>
       <c r="C59" s="15">
-        <f>0</f>
+        <f>History!$B$111</f>
         <v/>
       </c>
       <c r="D59" s="15">
@@ -15073,7 +15287,7 @@
         </is>
       </c>
       <c r="C78" s="15">
-        <f>161</f>
+        <f>History!$B$109</f>
         <v/>
       </c>
       <c r="D78" s="15">
@@ -15269,7 +15483,7 @@
         </is>
       </c>
       <c r="C85" s="15">
-        <f>91</f>
+        <f>History!$B$108</f>
         <v/>
       </c>
       <c r="D85" s="15">
@@ -15345,7 +15559,7 @@
         </is>
       </c>
       <c r="C88" s="15">
-        <f>705</f>
+        <f>History!$B$110</f>
         <v/>
       </c>
       <c r="D88" s="15">
@@ -15373,7 +15587,7 @@
         </is>
       </c>
       <c r="C89" s="15">
-        <f>0</f>
+        <f>History!$B$111</f>
         <v/>
       </c>
       <c r="D89" s="15">
@@ -15494,7 +15708,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>FCF bridge from WS07. Share count: buybacks and RSU issuance at a price growing 5% a year, 35% of SBC withheld for tax. Net cash starts at the 30 Jun 2026 actual.</t>
+          <t>FCF bridge from WS07. Share count: buybacks and RSU issuance at a price growing 5% a year, 35% of SBC withheld for tax. Both roll-forwards start from the same 2Q26 actual (net cash $9,593M, 597M diluted shares) and both consume the SAME flows: for FY2026 only the 2H26 buyback (FY26 less the 1H26 actual $2,139M) and only 2H26 SBC (FY26 less the 1H26 actual $897M); FY2027 and FY2028 take the full year. WS17 finding 3 (the FY2026 share roll applied the FULL-YEAR buyback and SBC to a 30 Jun 2026 count, double-counting the 1H26 repurchase and understating FY2026E shares by 8.55M) was fixed by WS18 here and in 13_driver_model.py. See research/notes/overnight/18_corrections-applied.md.</t>
         </is>
       </c>
     </row>
@@ -15583,7 +15797,7 @@
         </is>
       </c>
       <c r="C7" s="15">
-        <f>705</f>
+        <f>History!$B$110</f>
         <v/>
       </c>
       <c r="D7" s="15">
@@ -15611,7 +15825,7 @@
         </is>
       </c>
       <c r="C8" s="15">
-        <f>0</f>
+        <f>-History!$B$111</f>
         <v/>
       </c>
       <c r="D8" s="15">
@@ -15639,7 +15853,7 @@
         </is>
       </c>
       <c r="C9" s="15">
-        <f>-112</f>
+        <f>History!$B$112</f>
         <v/>
       </c>
       <c r="D9" s="15">
@@ -15667,7 +15881,7 @@
         </is>
       </c>
       <c r="C10" s="15">
-        <f>-232</f>
+        <f>History!$B$113</f>
         <v/>
       </c>
       <c r="D10" s="15">
@@ -15695,7 +15909,7 @@
         </is>
       </c>
       <c r="C11" s="15">
-        <f>127</f>
+        <f>History!$B$114</f>
         <v/>
       </c>
       <c r="D11" s="15">
@@ -15723,7 +15937,7 @@
         </is>
       </c>
       <c r="C12" s="15">
-        <f>-139</f>
+        <f>History!$B$115</f>
         <v/>
       </c>
       <c r="D12" s="15">
@@ -15751,7 +15965,7 @@
         </is>
       </c>
       <c r="C13" s="15">
-        <f>-33</f>
+        <f>History!$B$116</f>
         <v/>
       </c>
       <c r="D13" s="15">
@@ -15971,7 +16185,7 @@
         </is>
       </c>
       <c r="C21" s="15">
-        <f>3789</f>
+        <f>History!$B$117</f>
         <v/>
       </c>
       <c r="D21" s="15">
@@ -15999,7 +16213,7 @@
         </is>
       </c>
       <c r="C22" s="15">
-        <f>561</f>
+        <f>History!$B$118</f>
         <v/>
       </c>
       <c r="D22" s="15">
@@ -16018,7 +16232,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Diluted shares, period end</t>
+          <t>Diluted shares, period end (FY2025A col = the 2Q26 actual)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -16031,7 +16245,7 @@
         <v/>
       </c>
       <c r="D23" s="19">
-        <f>C23-D21/D20+D17/D20*(1-Inputs!$C$18)</f>
+        <f>C23-(D21-History!$B$48)/D20+(D17-History!$B$50)/D20*(1-Inputs!$C$18)</f>
         <v/>
       </c>
       <c r="E23" s="19">
@@ -16118,7 +16332,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Net cash ex float, period end</t>
+          <t>Net cash ex float, period end (FY2025A col = the 30 Jun 2026 actual)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -16228,7 +16442,7 @@
         </is>
       </c>
       <c r="C32" s="15">
-        <f>705</f>
+        <f>History!$B$110</f>
         <v/>
       </c>
       <c r="D32" s="15">
@@ -16256,7 +16470,7 @@
         </is>
       </c>
       <c r="C33" s="15">
-        <f>0</f>
+        <f>-History!$B$111</f>
         <v/>
       </c>
       <c r="D33" s="15">
@@ -16284,7 +16498,7 @@
         </is>
       </c>
       <c r="C34" s="15">
-        <f>-112</f>
+        <f>History!$B$112</f>
         <v/>
       </c>
       <c r="D34" s="15">
@@ -16312,7 +16526,7 @@
         </is>
       </c>
       <c r="C35" s="15">
-        <f>-232</f>
+        <f>History!$B$113</f>
         <v/>
       </c>
       <c r="D35" s="15">
@@ -16340,7 +16554,7 @@
         </is>
       </c>
       <c r="C36" s="15">
-        <f>127</f>
+        <f>History!$B$114</f>
         <v/>
       </c>
       <c r="D36" s="15">
@@ -16368,7 +16582,7 @@
         </is>
       </c>
       <c r="C37" s="15">
-        <f>-139</f>
+        <f>History!$B$115</f>
         <v/>
       </c>
       <c r="D37" s="15">
@@ -16396,7 +16610,7 @@
         </is>
       </c>
       <c r="C38" s="15">
-        <f>-33</f>
+        <f>History!$B$116</f>
         <v/>
       </c>
       <c r="D38" s="15">
@@ -16616,7 +16830,7 @@
         </is>
       </c>
       <c r="C46" s="15">
-        <f>3789</f>
+        <f>History!$B$117</f>
         <v/>
       </c>
       <c r="D46" s="15">
@@ -16644,7 +16858,7 @@
         </is>
       </c>
       <c r="C47" s="15">
-        <f>561</f>
+        <f>History!$B$118</f>
         <v/>
       </c>
       <c r="D47" s="15">
@@ -16663,7 +16877,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Diluted shares, period end</t>
+          <t>Diluted shares, period end (FY2025A col = the 2Q26 actual)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -16676,7 +16890,7 @@
         <v/>
       </c>
       <c r="D48" s="19">
-        <f>C48-D46/D45+D42/D45*(1-Inputs!$D$18)</f>
+        <f>C48-(D46-History!$B$48)/D45+(D42-History!$B$50)/D45*(1-Inputs!$D$18)</f>
         <v/>
       </c>
       <c r="E48" s="19">
@@ -16763,7 +16977,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Net cash ex float, period end</t>
+          <t>Net cash ex float, period end (FY2025A col = the 30 Jun 2026 actual)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -16873,7 +17087,7 @@
         </is>
       </c>
       <c r="C57" s="15">
-        <f>705</f>
+        <f>History!$B$110</f>
         <v/>
       </c>
       <c r="D57" s="15">
@@ -16901,7 +17115,7 @@
         </is>
       </c>
       <c r="C58" s="15">
-        <f>0</f>
+        <f>-History!$B$111</f>
         <v/>
       </c>
       <c r="D58" s="15">
@@ -16929,7 +17143,7 @@
         </is>
       </c>
       <c r="C59" s="15">
-        <f>-112</f>
+        <f>History!$B$112</f>
         <v/>
       </c>
       <c r="D59" s="15">
@@ -16957,7 +17171,7 @@
         </is>
       </c>
       <c r="C60" s="15">
-        <f>-232</f>
+        <f>History!$B$113</f>
         <v/>
       </c>
       <c r="D60" s="15">
@@ -16985,7 +17199,7 @@
         </is>
       </c>
       <c r="C61" s="15">
-        <f>127</f>
+        <f>History!$B$114</f>
         <v/>
       </c>
       <c r="D61" s="15">
@@ -17013,7 +17227,7 @@
         </is>
       </c>
       <c r="C62" s="15">
-        <f>-139</f>
+        <f>History!$B$115</f>
         <v/>
       </c>
       <c r="D62" s="15">
@@ -17041,7 +17255,7 @@
         </is>
       </c>
       <c r="C63" s="15">
-        <f>-33</f>
+        <f>History!$B$116</f>
         <v/>
       </c>
       <c r="D63" s="15">
@@ -17261,7 +17475,7 @@
         </is>
       </c>
       <c r="C71" s="15">
-        <f>3789</f>
+        <f>History!$B$117</f>
         <v/>
       </c>
       <c r="D71" s="15">
@@ -17289,7 +17503,7 @@
         </is>
       </c>
       <c r="C72" s="15">
-        <f>561</f>
+        <f>History!$B$118</f>
         <v/>
       </c>
       <c r="D72" s="15">
@@ -17308,7 +17522,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Diluted shares, period end</t>
+          <t>Diluted shares, period end (FY2025A col = the 2Q26 actual)</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -17321,7 +17535,7 @@
         <v/>
       </c>
       <c r="D73" s="19">
-        <f>C73-D71/D70+D67/D70*(1-Inputs!$E$18)</f>
+        <f>C73-(D71-History!$B$48)/D70+(D67-History!$B$50)/D70*(1-Inputs!$E$18)</f>
         <v/>
       </c>
       <c r="E73" s="19">
@@ -17408,7 +17622,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Net cash ex float, period end</t>
+          <t>Net cash ex float, period end (FY2025A col = the 30 Jun 2026 actual)</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -17444,7 +17658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -17506,6 +17720,11 @@
           <t>Bull</t>
         </is>
       </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Active (Inputs!B4)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -17525,6 +17744,10 @@
         <f>Costs!$E$81</f>
         <v/>
       </c>
+      <c r="E6" s="21">
+        <f>CHOOSE(Inputs!$B$4,B6,C6,D6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -17544,6 +17767,10 @@
         <f>Cash!$E$64</f>
         <v/>
       </c>
+      <c r="E7" s="21">
+        <f>CHOOSE(Inputs!$B$4,B7,C7,D7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -17563,6 +17790,10 @@
         <f>Cash!$E$68</f>
         <v/>
       </c>
+      <c r="E8" s="21">
+        <f>CHOOSE(Inputs!$B$4,B8,C8,D8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -17582,6 +17813,10 @@
         <f>Cash!$E$76</f>
         <v/>
       </c>
+      <c r="E9" s="9">
+        <f>CHOOSE(Inputs!$B$4,B9,C9,D9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -17601,6 +17836,10 @@
         <f>Cash!$E$77</f>
         <v/>
       </c>
+      <c r="E10" s="21">
+        <f>CHOOSE(Inputs!$B$4,B10,C10,D10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -17620,6 +17859,10 @@
         <f>Cash!$E$73</f>
         <v/>
       </c>
+      <c r="E11" s="15">
+        <f>CHOOSE(Inputs!$B$4,B11,C11,D11)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -17639,6 +17882,10 @@
         <f>Costs!$F$81</f>
         <v/>
       </c>
+      <c r="E12" s="21">
+        <f>CHOOSE(Inputs!$B$4,B12,C12,D12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -17658,6 +17905,10 @@
         <f>Cash!$F$77</f>
         <v/>
       </c>
+      <c r="E13" s="21">
+        <f>CHOOSE(Inputs!$B$4,B13,C13,D13)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -17677,6 +17928,10 @@
         <f>Cash!$F$73</f>
         <v/>
       </c>
+      <c r="E14" s="15">
+        <f>CHOOSE(Inputs!$B$4,B14,C14,D14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -17694,6 +17949,10 @@
       </c>
       <c r="D15" s="21">
         <f>Cash!$F$64</f>
+        <v/>
+      </c>
+      <c r="E15" s="21">
+        <f>CHOOSE(Inputs!$B$4,B15,C15,D15)</f>
         <v/>
       </c>
     </row>
@@ -17733,6 +17992,11 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
+          <t>Active (Inputs!B4)</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
           <t>Multiple source</t>
         </is>
       </c>
@@ -17755,7 +18019,11 @@
         <f>(Inputs!$E$14*D6+D10)/D11</f>
         <v/>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="24">
+        <f>CHOOSE(Inputs!$B$4,B19,C19,D19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>WS12 13.5 / 16.5 / 18.5x</t>
         </is>
@@ -17779,7 +18047,11 @@
         <f>(Inputs!$E$15*D7+D10)/D11</f>
         <v/>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="24">
+        <f>CHOOSE(Inputs!$B$4,B20,C20,D20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>5 Sep 15/19/23x rescaled by WS12's 0.75x haircut</t>
         </is>
@@ -17803,7 +18075,11 @@
         <f>Inputs!$E$16*D8/D11</f>
         <v/>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="24">
+        <f>CHOOSE(Inputs!$B$4,B21,C21,D21)</f>
+        <v/>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>same 0.75x haircut on 20/26/32x</t>
         </is>
@@ -17827,7 +18103,11 @@
         <f>Inputs!$E$17*D9</f>
         <v/>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" s="24">
+        <f>CHOOSE(Inputs!$B$4,B22,C22,D22)</f>
+        <v/>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>same</t>
         </is>
@@ -17851,7 +18131,11 @@
         <f>(Inputs!$E$14*D12+D13)/D14</f>
         <v/>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" s="24">
+        <f>CHOOSE(Inputs!$B$4,B23,C23,D23)</f>
+        <v/>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>WS12 multiples on the FY28 basis</t>
         </is>
@@ -17917,27 +18201,27 @@
         <v>1</v>
       </c>
       <c r="B27" s="21">
-        <f>B7*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*0/9))</f>
+        <f>B7*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*($A27-1)/9))</f>
         <v/>
       </c>
       <c r="C27" s="21">
-        <f>C7*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*0/9))</f>
+        <f>C7*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*($A27-1)/9))</f>
         <v/>
       </c>
       <c r="D27" s="21">
-        <f>D7*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*0/9))</f>
+        <f>D7*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*($A27-1)/9))</f>
         <v/>
       </c>
       <c r="E27" s="21">
-        <f>B27/(1+Inputs!$C$11)^1</f>
+        <f>B27/(1+Inputs!$C$11)^$A27</f>
         <v/>
       </c>
       <c r="F27" s="21">
-        <f>C27/(1+Inputs!$D$11)^1</f>
+        <f>C27/(1+Inputs!$D$11)^$A27</f>
         <v/>
       </c>
       <c r="G27" s="21">
-        <f>D27/(1+Inputs!$E$11)^1</f>
+        <f>D27/(1+Inputs!$E$11)^$A27</f>
         <v/>
       </c>
     </row>
@@ -17946,27 +18230,27 @@
         <v>2</v>
       </c>
       <c r="B28" s="21">
-        <f>B27*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*1/9))</f>
+        <f>B27*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*($A28-1)/9))</f>
         <v/>
       </c>
       <c r="C28" s="21">
-        <f>C27*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*1/9))</f>
+        <f>C27*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*($A28-1)/9))</f>
         <v/>
       </c>
       <c r="D28" s="21">
-        <f>D27*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*1/9))</f>
+        <f>D27*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*($A28-1)/9))</f>
         <v/>
       </c>
       <c r="E28" s="21">
-        <f>B28/(1+Inputs!$C$11)^2</f>
+        <f>B28/(1+Inputs!$C$11)^$A28</f>
         <v/>
       </c>
       <c r="F28" s="21">
-        <f>C28/(1+Inputs!$D$11)^2</f>
+        <f>C28/(1+Inputs!$D$11)^$A28</f>
         <v/>
       </c>
       <c r="G28" s="21">
-        <f>D28/(1+Inputs!$E$11)^2</f>
+        <f>D28/(1+Inputs!$E$11)^$A28</f>
         <v/>
       </c>
     </row>
@@ -17975,27 +18259,27 @@
         <v>3</v>
       </c>
       <c r="B29" s="21">
-        <f>B28*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*2/9))</f>
+        <f>B28*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*($A29-1)/9))</f>
         <v/>
       </c>
       <c r="C29" s="21">
-        <f>C28*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*2/9))</f>
+        <f>C28*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*($A29-1)/9))</f>
         <v/>
       </c>
       <c r="D29" s="21">
-        <f>D28*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*2/9))</f>
+        <f>D28*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*($A29-1)/9))</f>
         <v/>
       </c>
       <c r="E29" s="21">
-        <f>B29/(1+Inputs!$C$11)^3</f>
+        <f>B29/(1+Inputs!$C$11)^$A29</f>
         <v/>
       </c>
       <c r="F29" s="21">
-        <f>C29/(1+Inputs!$D$11)^3</f>
+        <f>C29/(1+Inputs!$D$11)^$A29</f>
         <v/>
       </c>
       <c r="G29" s="21">
-        <f>D29/(1+Inputs!$E$11)^3</f>
+        <f>D29/(1+Inputs!$E$11)^$A29</f>
         <v/>
       </c>
     </row>
@@ -18004,27 +18288,27 @@
         <v>4</v>
       </c>
       <c r="B30" s="21">
-        <f>B29*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*3/9))</f>
+        <f>B29*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*($A30-1)/9))</f>
         <v/>
       </c>
       <c r="C30" s="21">
-        <f>C29*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*3/9))</f>
+        <f>C29*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*($A30-1)/9))</f>
         <v/>
       </c>
       <c r="D30" s="21">
-        <f>D29*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*3/9))</f>
+        <f>D29*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*($A30-1)/9))</f>
         <v/>
       </c>
       <c r="E30" s="21">
-        <f>B30/(1+Inputs!$C$11)^4</f>
+        <f>B30/(1+Inputs!$C$11)^$A30</f>
         <v/>
       </c>
       <c r="F30" s="21">
-        <f>C30/(1+Inputs!$D$11)^4</f>
+        <f>C30/(1+Inputs!$D$11)^$A30</f>
         <v/>
       </c>
       <c r="G30" s="21">
-        <f>D30/(1+Inputs!$E$11)^4</f>
+        <f>D30/(1+Inputs!$E$11)^$A30</f>
         <v/>
       </c>
     </row>
@@ -18033,27 +18317,27 @@
         <v>5</v>
       </c>
       <c r="B31" s="21">
-        <f>B30*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*4/9))</f>
+        <f>B30*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*($A31-1)/9))</f>
         <v/>
       </c>
       <c r="C31" s="21">
-        <f>C30*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*4/9))</f>
+        <f>C30*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*($A31-1)/9))</f>
         <v/>
       </c>
       <c r="D31" s="21">
-        <f>D30*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*4/9))</f>
+        <f>D30*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*($A31-1)/9))</f>
         <v/>
       </c>
       <c r="E31" s="21">
-        <f>B31/(1+Inputs!$C$11)^5</f>
+        <f>B31/(1+Inputs!$C$11)^$A31</f>
         <v/>
       </c>
       <c r="F31" s="21">
-        <f>C31/(1+Inputs!$D$11)^5</f>
+        <f>C31/(1+Inputs!$D$11)^$A31</f>
         <v/>
       </c>
       <c r="G31" s="21">
-        <f>D31/(1+Inputs!$E$11)^5</f>
+        <f>D31/(1+Inputs!$E$11)^$A31</f>
         <v/>
       </c>
     </row>
@@ -18062,27 +18346,27 @@
         <v>6</v>
       </c>
       <c r="B32" s="21">
-        <f>B31*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*5/9))</f>
+        <f>B31*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*($A32-1)/9))</f>
         <v/>
       </c>
       <c r="C32" s="21">
-        <f>C31*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*5/9))</f>
+        <f>C31*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*($A32-1)/9))</f>
         <v/>
       </c>
       <c r="D32" s="21">
-        <f>D31*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*5/9))</f>
+        <f>D31*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*($A32-1)/9))</f>
         <v/>
       </c>
       <c r="E32" s="21">
-        <f>B32/(1+Inputs!$C$11)^6</f>
+        <f>B32/(1+Inputs!$C$11)^$A32</f>
         <v/>
       </c>
       <c r="F32" s="21">
-        <f>C32/(1+Inputs!$D$11)^6</f>
+        <f>C32/(1+Inputs!$D$11)^$A32</f>
         <v/>
       </c>
       <c r="G32" s="21">
-        <f>D32/(1+Inputs!$E$11)^6</f>
+        <f>D32/(1+Inputs!$E$11)^$A32</f>
         <v/>
       </c>
     </row>
@@ -18091,27 +18375,27 @@
         <v>7</v>
       </c>
       <c r="B33" s="21">
-        <f>B32*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*6/9))</f>
+        <f>B32*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*($A33-1)/9))</f>
         <v/>
       </c>
       <c r="C33" s="21">
-        <f>C32*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*6/9))</f>
+        <f>C32*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*($A33-1)/9))</f>
         <v/>
       </c>
       <c r="D33" s="21">
-        <f>D32*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*6/9))</f>
+        <f>D32*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*($A33-1)/9))</f>
         <v/>
       </c>
       <c r="E33" s="21">
-        <f>B33/(1+Inputs!$C$11)^7</f>
+        <f>B33/(1+Inputs!$C$11)^$A33</f>
         <v/>
       </c>
       <c r="F33" s="21">
-        <f>C33/(1+Inputs!$D$11)^7</f>
+        <f>C33/(1+Inputs!$D$11)^$A33</f>
         <v/>
       </c>
       <c r="G33" s="21">
-        <f>D33/(1+Inputs!$E$11)^7</f>
+        <f>D33/(1+Inputs!$E$11)^$A33</f>
         <v/>
       </c>
     </row>
@@ -18120,27 +18404,27 @@
         <v>8</v>
       </c>
       <c r="B34" s="21">
-        <f>B33*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*7/9))</f>
+        <f>B33*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*($A34-1)/9))</f>
         <v/>
       </c>
       <c r="C34" s="21">
-        <f>C33*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*7/9))</f>
+        <f>C33*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*($A34-1)/9))</f>
         <v/>
       </c>
       <c r="D34" s="21">
-        <f>D33*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*7/9))</f>
+        <f>D33*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*($A34-1)/9))</f>
         <v/>
       </c>
       <c r="E34" s="21">
-        <f>B34/(1+Inputs!$C$11)^8</f>
+        <f>B34/(1+Inputs!$C$11)^$A34</f>
         <v/>
       </c>
       <c r="F34" s="21">
-        <f>C34/(1+Inputs!$D$11)^8</f>
+        <f>C34/(1+Inputs!$D$11)^$A34</f>
         <v/>
       </c>
       <c r="G34" s="21">
-        <f>D34/(1+Inputs!$E$11)^8</f>
+        <f>D34/(1+Inputs!$E$11)^$A34</f>
         <v/>
       </c>
     </row>
@@ -18149,27 +18433,27 @@
         <v>9</v>
       </c>
       <c r="B35" s="21">
-        <f>B34*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*8/9))</f>
+        <f>B34*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*($A35-1)/9))</f>
         <v/>
       </c>
       <c r="C35" s="21">
-        <f>C34*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*8/9))</f>
+        <f>C34*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*($A35-1)/9))</f>
         <v/>
       </c>
       <c r="D35" s="21">
-        <f>D34*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*8/9))</f>
+        <f>D34*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*($A35-1)/9))</f>
         <v/>
       </c>
       <c r="E35" s="21">
-        <f>B35/(1+Inputs!$C$11)^9</f>
+        <f>B35/(1+Inputs!$C$11)^$A35</f>
         <v/>
       </c>
       <c r="F35" s="21">
-        <f>C35/(1+Inputs!$D$11)^9</f>
+        <f>C35/(1+Inputs!$D$11)^$A35</f>
         <v/>
       </c>
       <c r="G35" s="21">
-        <f>D35/(1+Inputs!$E$11)^9</f>
+        <f>D35/(1+Inputs!$E$11)^$A35</f>
         <v/>
       </c>
     </row>
@@ -18178,27 +18462,27 @@
         <v>10</v>
       </c>
       <c r="B36" s="21">
-        <f>B35*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*9/9))</f>
+        <f>B35*(1+(Inputs!$C$13+(Inputs!$C$12-Inputs!$C$13)*($A36-1)/9))</f>
         <v/>
       </c>
       <c r="C36" s="21">
-        <f>C35*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*9/9))</f>
+        <f>C35*(1+(Inputs!$D$13+(Inputs!$D$12-Inputs!$D$13)*($A36-1)/9))</f>
         <v/>
       </c>
       <c r="D36" s="21">
-        <f>D35*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*9/9))</f>
+        <f>D35*(1+(Inputs!$E$13+(Inputs!$E$12-Inputs!$E$13)*($A36-1)/9))</f>
         <v/>
       </c>
       <c r="E36" s="21">
-        <f>B36/(1+Inputs!$C$11)^10</f>
+        <f>B36/(1+Inputs!$C$11)^$A36</f>
         <v/>
       </c>
       <c r="F36" s="21">
-        <f>C36/(1+Inputs!$D$11)^10</f>
+        <f>C36/(1+Inputs!$D$11)^$A36</f>
         <v/>
       </c>
       <c r="G36" s="21">
-        <f>D36/(1+Inputs!$E$11)^10</f>
+        <f>D36/(1+Inputs!$E$11)^$A36</f>
         <v/>
       </c>
     </row>
@@ -18209,15 +18493,15 @@
         </is>
       </c>
       <c r="E37" s="21">
-        <f>B36*(1+Inputs!$C$12)/(Inputs!$C$11-Inputs!$C$12)/(1+Inputs!$C$11)^10</f>
+        <f>B36*(1+Inputs!$C$12)/(Inputs!$C$11-Inputs!$C$12)/(1+Inputs!$C$11)^$A36</f>
         <v/>
       </c>
       <c r="F37" s="21">
-        <f>C36*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10</f>
+        <f>C36*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^$A36</f>
         <v/>
       </c>
       <c r="G37" s="21">
-        <f>D36*(1+Inputs!$E$12)/(Inputs!$E$11-Inputs!$E$12)/(1+Inputs!$E$11)^10</f>
+        <f>D36*(1+Inputs!$E$12)/(Inputs!$E$11-Inputs!$E$12)/(1+Inputs!$E$11)^$A36</f>
         <v/>
       </c>
     </row>
@@ -18257,6 +18541,15 @@
       <c r="D39" s="24">
         <f>(G38+D10)/D11</f>
         <v/>
+      </c>
+      <c r="E39" s="24">
+        <f>CHOOSE(Inputs!$B$4,B39,C39,D39)</f>
+        <v/>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>column E on this row is the Active (Inputs!B4) selection, not a PV</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -18293,6 +18586,11 @@
           <t>Bull</t>
         </is>
       </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Active (Inputs!B4)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -18312,6 +18610,10 @@
         <f>MIN(D19,D20,D21,D22,D23,D39)</f>
         <v/>
       </c>
+      <c r="E43" s="24">
+        <f>CHOOSE(Inputs!$B$4,B43,C43,D43)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -18331,6 +18633,10 @@
         <f>MAX(D19,D20,D21,D22,D23,D39)</f>
         <v/>
       </c>
+      <c r="E44" s="24">
+        <f>CHOOSE(Inputs!$B$4,B44,C44,D44)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -18350,6 +18656,10 @@
         <f>AVERAGE(D19,D20,D21,D22,D23,D39)</f>
         <v/>
       </c>
+      <c r="E45" s="24">
+        <f>CHOOSE(Inputs!$B$4,B45,C45,D45)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -18369,6 +18679,10 @@
         <f>Inputs!$E$8</f>
         <v/>
       </c>
+      <c r="E46" s="9">
+        <f>CHOOSE(Inputs!$B$4,B46,C46,D46)</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -18388,6 +18702,10 @@
         <f>D43/D46-1</f>
         <v/>
       </c>
+      <c r="E47" s="23">
+        <f>E43/E46-1</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -18407,6 +18725,10 @@
         <f>D44/D46-1</f>
         <v/>
       </c>
+      <c r="E48" s="23">
+        <f>E44/E46-1</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -18424,6 +18746,10 @@
       </c>
       <c r="D49" s="23">
         <f>D45/D46-1</f>
+        <v/>
+      </c>
+      <c r="E49" s="23">
+        <f>E45/E46-1</f>
         <v/>
       </c>
     </row>
@@ -18487,11 +18813,11 @@
         <v>0.03</v>
       </c>
       <c r="B54" s="9">
-        <f>(History!$B$102*(1+A54)/(Inputs!$D$11-A54)*(1-((1+A54)/(1+Inputs!$D$11))^10)+History!$B$102*(1+A54)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>(History!$B$103*(1+A54)/(Inputs!$D$11-A54)*(1-((1+A54)/(1+Inputs!$D$11))^10)+History!$B$103*(1+A54)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
       <c r="C54" s="9">
-        <f>((History!$B$102-History!$B$103)*(1+A54)/(Inputs!$D$11-A54)*(1-((1+A54)/(1+Inputs!$D$11))^10)+(History!$B$102-History!$B$103)*(1+A54)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>((History!$B$103-History!$B$104)*(1+A54)/(Inputs!$D$11-A54)*(1-((1+A54)/(1+Inputs!$D$11))^10)+(History!$B$103-History!$B$104)*(1+A54)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
     </row>
@@ -18500,11 +18826,11 @@
         <v>0.05</v>
       </c>
       <c r="B55" s="9">
-        <f>(History!$B$102*(1+A55)/(Inputs!$D$11-A55)*(1-((1+A55)/(1+Inputs!$D$11))^10)+History!$B$102*(1+A55)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>(History!$B$103*(1+A55)/(Inputs!$D$11-A55)*(1-((1+A55)/(1+Inputs!$D$11))^10)+History!$B$103*(1+A55)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
       <c r="C55" s="9">
-        <f>((History!$B$102-History!$B$103)*(1+A55)/(Inputs!$D$11-A55)*(1-((1+A55)/(1+Inputs!$D$11))^10)+(History!$B$102-History!$B$103)*(1+A55)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>((History!$B$103-History!$B$104)*(1+A55)/(Inputs!$D$11-A55)*(1-((1+A55)/(1+Inputs!$D$11))^10)+(History!$B$103-History!$B$104)*(1+A55)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
     </row>
@@ -18513,11 +18839,11 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="B56" s="9">
-        <f>(History!$B$102*(1+A56)/(Inputs!$D$11-A56)*(1-((1+A56)/(1+Inputs!$D$11))^10)+History!$B$102*(1+A56)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>(History!$B$103*(1+A56)/(Inputs!$D$11-A56)*(1-((1+A56)/(1+Inputs!$D$11))^10)+History!$B$103*(1+A56)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
       <c r="C56" s="9">
-        <f>((History!$B$102-History!$B$103)*(1+A56)/(Inputs!$D$11-A56)*(1-((1+A56)/(1+Inputs!$D$11))^10)+(History!$B$102-History!$B$103)*(1+A56)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>((History!$B$103-History!$B$104)*(1+A56)/(Inputs!$D$11-A56)*(1-((1+A56)/(1+Inputs!$D$11))^10)+(History!$B$103-History!$B$104)*(1+A56)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
     </row>
@@ -18526,11 +18852,11 @@
         <v>0.075</v>
       </c>
       <c r="B57" s="9">
-        <f>(History!$B$102*(1+A57)/(Inputs!$D$11-A57)*(1-((1+A57)/(1+Inputs!$D$11))^10)+History!$B$102*(1+A57)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>(History!$B$103*(1+A57)/(Inputs!$D$11-A57)*(1-((1+A57)/(1+Inputs!$D$11))^10)+History!$B$103*(1+A57)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
       <c r="C57" s="9">
-        <f>((History!$B$102-History!$B$103)*(1+A57)/(Inputs!$D$11-A57)*(1-((1+A57)/(1+Inputs!$D$11))^10)+(History!$B$102-History!$B$103)*(1+A57)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>((History!$B$103-History!$B$104)*(1+A57)/(Inputs!$D$11-A57)*(1-((1+A57)/(1+Inputs!$D$11))^10)+(History!$B$103-History!$B$104)*(1+A57)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
     </row>
@@ -18539,11 +18865,11 @@
         <v>0.09</v>
       </c>
       <c r="B58" s="9">
-        <f>(History!$B$102*(1+A58)/(Inputs!$D$11-A58)*(1-((1+A58)/(1+Inputs!$D$11))^10)+History!$B$102*(1+A58)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>(History!$B$103*(1+A58)/(Inputs!$D$11-A58)*(1-((1+A58)/(1+Inputs!$D$11))^10)+History!$B$103*(1+A58)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
       <c r="C58" s="9">
-        <f>((History!$B$102-History!$B$103)*(1+A58)/(Inputs!$D$11-A58)*(1-((1+A58)/(1+Inputs!$D$11))^10)+(History!$B$102-History!$B$103)*(1+A58)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>((History!$B$103-History!$B$104)*(1+A58)/(Inputs!$D$11-A58)*(1-((1+A58)/(1+Inputs!$D$11))^10)+(History!$B$103-History!$B$104)*(1+A58)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
     </row>
@@ -18552,11 +18878,11 @@
         <v>0.11</v>
       </c>
       <c r="B59" s="9">
-        <f>(History!$B$102*(1+A59)/(Inputs!$D$11-A59)*(1-((1+A59)/(1+Inputs!$D$11))^10)+History!$B$102*(1+A59)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>(History!$B$103*(1+A59)/(Inputs!$D$11-A59)*(1-((1+A59)/(1+Inputs!$D$11))^10)+History!$B$103*(1+A59)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
       <c r="C59" s="9">
-        <f>((History!$B$102-History!$B$103)*(1+A59)/(Inputs!$D$11-A59)*(1-((1+A59)/(1+Inputs!$D$11))^10)+(History!$B$102-History!$B$103)*(1+A59)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>((History!$B$103-History!$B$104)*(1+A59)/(Inputs!$D$11-A59)*(1-((1+A59)/(1+Inputs!$D$11))^10)+(History!$B$103-History!$B$104)*(1+A59)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
     </row>
@@ -18565,11 +18891,11 @@
         <v>0.13</v>
       </c>
       <c r="B60" s="9">
-        <f>(History!$B$102*(1+A60)/(Inputs!$D$11-A60)*(1-((1+A60)/(1+Inputs!$D$11))^10)+History!$B$102*(1+A60)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>(History!$B$103*(1+A60)/(Inputs!$D$11-A60)*(1-((1+A60)/(1+Inputs!$D$11))^10)+History!$B$103*(1+A60)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
       <c r="C60" s="9">
-        <f>((History!$B$102-History!$B$103)*(1+A60)/(Inputs!$D$11-A60)*(1-((1+A60)/(1+Inputs!$D$11))^10)+(History!$B$102-History!$B$103)*(1+A60)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>((History!$B$103-History!$B$104)*(1+A60)/(Inputs!$D$11-A60)*(1-((1+A60)/(1+Inputs!$D$11))^10)+(History!$B$103-History!$B$104)*(1+A60)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
     </row>
@@ -18578,11 +18904,11 @@
         <v>0.135</v>
       </c>
       <c r="B61" s="9">
-        <f>(History!$B$102*(1+A61)/(Inputs!$D$11-A61)*(1-((1+A61)/(1+Inputs!$D$11))^10)+History!$B$102*(1+A61)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>(History!$B$103*(1+A61)/(Inputs!$D$11-A61)*(1-((1+A61)/(1+Inputs!$D$11))^10)+History!$B$103*(1+A61)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
       <c r="C61" s="9">
-        <f>((History!$B$102-History!$B$103)*(1+A61)/(Inputs!$D$11-A61)*(1-((1+A61)/(1+Inputs!$D$11))^10)+(History!$B$102-History!$B$103)*(1+A61)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>((History!$B$103-History!$B$104)*(1+A61)/(Inputs!$D$11-A61)*(1-((1+A61)/(1+Inputs!$D$11))^10)+(History!$B$103-History!$B$104)*(1+A61)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
     </row>
@@ -18591,11 +18917,11 @@
         <v>0.15</v>
       </c>
       <c r="B62" s="9">
-        <f>(History!$B$102*(1+A62)/(Inputs!$D$11-A62)*(1-((1+A62)/(1+Inputs!$D$11))^10)+History!$B$102*(1+A62)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>(History!$B$103*(1+A62)/(Inputs!$D$11-A62)*(1-((1+A62)/(1+Inputs!$D$11))^10)+History!$B$103*(1+A62)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
       <c r="C62" s="9">
-        <f>((History!$B$102-History!$B$103)*(1+A62)/(Inputs!$D$11-A62)*(1-((1+A62)/(1+Inputs!$D$11))^10)+(History!$B$102-History!$B$103)*(1+A62)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>((History!$B$103-History!$B$104)*(1+A62)/(Inputs!$D$11-A62)*(1-((1+A62)/(1+Inputs!$D$11))^10)+(History!$B$103-History!$B$104)*(1+A62)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
     </row>
@@ -18604,11 +18930,11 @@
         <v>0.17</v>
       </c>
       <c r="B63" s="9">
-        <f>(History!$B$102*(1+A63)/(Inputs!$D$11-A63)*(1-((1+A63)/(1+Inputs!$D$11))^10)+History!$B$102*(1+A63)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>(History!$B$103*(1+A63)/(Inputs!$D$11-A63)*(1-((1+A63)/(1+Inputs!$D$11))^10)+History!$B$103*(1+A63)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
       <c r="C63" s="9">
-        <f>((History!$B$102-History!$B$103)*(1+A63)/(Inputs!$D$11-A63)*(1-((1+A63)/(1+Inputs!$D$11))^10)+(History!$B$102-History!$B$103)*(1+A63)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
+        <f>((History!$B$103-History!$B$104)*(1+A63)/(Inputs!$D$11-A63)*(1-((1+A63)/(1+Inputs!$D$11))^10)+(History!$B$103-History!$B$104)*(1+A63)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10</f>
         <v/>
       </c>
     </row>
@@ -18618,10 +18944,10 @@
           <t>Solved implied 10-year growth at spot (constant growth, then terminal):</t>
         </is>
       </c>
-      <c r="B64" s="20" t="n">
+      <c r="B64" s="18" t="n">
         <v>0.08511676475842622</v>
       </c>
-      <c r="C64" s="20" t="n">
+      <c r="C64" s="18" t="n">
         <v>0.1441642817145657</v>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -18635,287 +18961,307 @@
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Check: value per share at the solved growth, less spot (0.00 = still current)</t>
+        </is>
+      </c>
+      <c r="B65" s="9">
+        <f>(History!$B$103*(1+B64)/(Inputs!$D$11-B64)*(1-((1+B64)/(1+Inputs!$D$11))^10)+History!$B$103*(1+B64)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10-Inputs!$D$8</f>
+        <v/>
+      </c>
+      <c r="C65" s="9">
+        <f>((History!$B$103-History!$B$104)*(1+C64)/(Inputs!$D$11-C64)*(1-((1+C64)/(1+Inputs!$D$11))^10)+(History!$B$103-History!$B$104)*(1+C64)^10*(1+Inputs!$D$12)/(Inputs!$D$11-Inputs!$D$12)/(1+Inputs!$D$11)^10+Inputs!$D$9)/Inputs!$D$10-Inputs!$D$8</f>
+        <v/>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>The solved cells above are yellow because they are an input, not a formula: a bisection run in analysis/src/overnight/13_driver_model.py. If this row stops reading 0.00, re-run that script - the cost of equity or the terminal growth moved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>6. SCENARIO GRID - FY2027E revenue growth x adj. EBITDA margin x exit multiple</t>
         </is>
       </c>
-      <c r="B66" s="6" t="n"/>
-      <c r="C66" s="6" t="n"/>
-      <c r="D66" s="6" t="n"/>
-      <c r="E66" s="6" t="n"/>
-      <c r="F66" s="6" t="n"/>
-      <c r="G66" s="6" t="n"/>
-      <c r="H66" s="6" t="n"/>
-      <c r="I66" s="6" t="n"/>
-      <c r="J66" s="6" t="n"/>
-      <c r="K66" s="6" t="n"/>
-      <c r="L66" s="6" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="B67" s="6" t="n"/>
+      <c r="C67" s="6" t="n"/>
+      <c r="D67" s="6" t="n"/>
+      <c r="E67" s="6" t="n"/>
+      <c r="F67" s="6" t="n"/>
+      <c r="G67" s="6" t="n"/>
+      <c r="H67" s="6" t="n"/>
+      <c r="I67" s="6" t="n"/>
+      <c r="J67" s="6" t="n"/>
+      <c r="K67" s="6" t="n"/>
+      <c r="L67" s="6" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>Price at the base exit multiple; rows = FY27 revenue growth, columns = FY27 margin</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="7" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
         <is>
           <t>Revenue growth \ margin</t>
         </is>
       </c>
-      <c r="B68" s="26" t="n">
+      <c r="B69" s="26" t="n">
         <v>0.32</v>
       </c>
-      <c r="C68" s="26" t="n">
+      <c r="C69" s="26" t="n">
         <v>0.34</v>
       </c>
-      <c r="D68" s="26" t="n">
+      <c r="D69" s="26" t="n">
         <v>0.355</v>
       </c>
-      <c r="E68" s="26" t="n">
+      <c r="E69" s="26" t="n">
         <v>0.365</v>
       </c>
-      <c r="F68" s="26" t="n">
+      <c r="F69" s="26" t="n">
         <v>0.375</v>
       </c>
-      <c r="G68" s="26" t="n">
+      <c r="G69" s="26" t="n">
         <v>0.39</v>
       </c>
-      <c r="H68" s="26" t="n">
+      <c r="H69" s="26" t="n">
         <v>0.41</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="20" t="n">
+    <row r="70">
+      <c r="A70" s="18" t="n">
         <v>0.04</v>
       </c>
-      <c r="B69" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.04)*0.32+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="C69" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.04)*0.34+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="D69" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.04)*0.355+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="E69" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.04)*0.365+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="F69" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.04)*0.375+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="G69" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.04)*0.39+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="H69" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.04)*0.41+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="20" t="n">
+      <c r="B70" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A70)*B$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="C70" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A70)*C$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="D70" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A70)*D$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="E70" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A70)*E$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="F70" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A70)*F$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="G70" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A70)*G$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="H70" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A70)*H$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="18" t="n">
         <v>0.06</v>
       </c>
-      <c r="B70" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.06)*0.32+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="C70" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.06)*0.34+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="D70" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.06)*0.355+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="E70" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.06)*0.365+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="F70" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.06)*0.375+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="G70" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.06)*0.39+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="H70" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.06)*0.41+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="20" t="n">
+      <c r="B71" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A71)*B$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="C71" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A71)*C$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="D71" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A71)*D$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="E71" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A71)*E$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="F71" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A71)*F$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="G71" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A71)*G$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="H71" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A71)*H$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="18" t="n">
         <v>0.08</v>
       </c>
-      <c r="B71" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.08)*0.32+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="C71" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.08)*0.34+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="D71" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.08)*0.355+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="E71" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.08)*0.365+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="F71" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.08)*0.375+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="G71" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.08)*0.39+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="H71" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.08)*0.41+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="20" t="n">
+      <c r="B72" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A72)*B$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="C72" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A72)*C$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="D72" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A72)*D$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="E72" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A72)*E$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="F72" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A72)*F$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="G72" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A72)*G$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="H72" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A72)*H$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="18" t="n">
         <v>0.1</v>
       </c>
-      <c r="B72" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.1)*0.32+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="C72" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.1)*0.34+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="D72" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.1)*0.355+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="E72" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.1)*0.365+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="F72" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.1)*0.375+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="G72" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.1)*0.39+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="H72" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.1)*0.41+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="20" t="n">
+      <c r="B73" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A73)*B$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="C73" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A73)*C$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="D73" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A73)*D$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="E73" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A73)*E$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="F73" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A73)*F$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="G73" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A73)*G$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="H73" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A73)*H$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="18" t="n">
         <v>0.12</v>
       </c>
-      <c r="B73" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.12)*0.32+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="C73" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.12)*0.34+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="D73" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.12)*0.355+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="E73" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.12)*0.365+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="F73" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.12)*0.375+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="G73" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.12)*0.39+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="H73" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.12)*0.41+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="20" t="n">
+      <c r="B74" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A74)*B$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="C74" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A74)*C$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="D74" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A74)*D$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="E74" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A74)*E$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="F74" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A74)*F$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="G74" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A74)*G$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="H74" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A74)*H$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="18" t="n">
         <v>0.14</v>
       </c>
-      <c r="B74" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.14)*0.32+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="C74" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.14)*0.34+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="D74" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.14)*0.355+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="E74" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.14)*0.365+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="F74" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.14)*0.375+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="G74" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.14)*0.39+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="H74" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.14)*0.41+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="20" t="n">
+      <c r="B75" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A75)*B$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="C75" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A75)*C$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="D75" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A75)*D$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="E75" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A75)*E$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="F75" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A75)*F$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="G75" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A75)*G$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="H75" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A75)*H$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="18" t="n">
         <v>0.16</v>
       </c>
-      <c r="B75" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.16)*0.32+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="C75" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.16)*0.34+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="D75" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.16)*0.355+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="E75" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.16)*0.365+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="F75" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.16)*0.375+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="G75" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.16)*0.39+Cash!$E$52)/Cash!$E$48</f>
-        <v/>
-      </c>
-      <c r="H75" s="9">
-        <f>(Inputs!$D$14*Revenue!$I$77*(1+0.16)*0.41+Cash!$E$52)/Cash!$E$48</f>
+      <c r="B76" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A76)*B$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="C76" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A76)*C$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="D76" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A76)*D$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="E76" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A76)*E$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="F76" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A76)*F$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="G76" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A76)*G$69+Cash!$E$52)/Cash!$E$48</f>
+        <v/>
+      </c>
+      <c r="H76" s="9">
+        <f>(Inputs!$D$14*Revenue!$I$77*(1+$A76)*H$69+Cash!$E$52)/Cash!$E$48</f>
         <v/>
       </c>
     </row>
@@ -18939,8 +19285,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19442,7 +19787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -19465,7 +19810,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Model columns are live formulas off the Revenue and Costs sheets. External bars are constants with their source. Q3 2026 reports 5 Nov 2026 (Zacks expected date).</t>
+          <t>Model columns are live formulas off the Revenue and Costs sheets; the Active column follows the scenario selector on Inputs!B4. External bars are constants with their source. Q3 2026 reports 5 Nov 2026 (Zacks expected date).</t>
         </is>
       </c>
     </row>
@@ -19492,15 +19837,20 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
+          <t>Active (Inputs!B4)</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
           <t>Company guide</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Street / cushion bar</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Source of the bar</t>
         </is>
@@ -19524,17 +19874,21 @@
         <f>Revenue!$C$118</f>
         <v/>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="22">
+        <f>CHOOSE(Inputs!$B$4,B5,C5,D5)</f>
+        <v/>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>$4,690-4,770m (+15-17%)</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Street $4,740m; cushion-adj $4,815m</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>2Q26 letter; WS04 Zacks 7 est; WS02 02_q3_2026_guide_card.csv (last-8 median cushion +1.79%)</t>
         </is>
@@ -19558,17 +19912,21 @@
         <f>Revenue!$C$119</f>
         <v/>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="23">
+        <f>CHOOSE(Inputs!$B$4,B6,C6,D6)</f>
+        <v/>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>+15% to +17%</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>+15.79% (Street)</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>WS02, WS04</t>
         </is>
@@ -19592,17 +19950,21 @@
         <f>Revenue!$C$104</f>
         <v/>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="19">
+        <f>CHOOSE(Inputs!$B$4,B7,C7,D7)</f>
+        <v/>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>low double-digit growth</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>144-146m (derived)</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>WS04 04_q3_2026_breakeven.csv; WS02 puts the cushion-adjusted range at 150-154m</t>
         </is>
@@ -19626,17 +19988,21 @@
         <f>Revenue!$C$105</f>
         <v/>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="23">
+        <f>CHOOSE(Inputs!$B$4,B8,C8,D8)</f>
+        <v/>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>'low double digit' (10-12%)</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>WS08 nowcast +12.1% (9.3-14.9)</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>WS08 08_q3_2026_nowcast.csv demand_eq; naive baseline +10.3%</t>
         </is>
@@ -19660,17 +20026,21 @@
         <f>Revenue!$C$108</f>
         <v/>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="24">
+        <f>CHOOSE(Inputs!$B$4,B9,C9,D9)</f>
+        <v/>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>'up moderately'</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>2Q26 letter</t>
         </is>
@@ -19694,17 +20064,21 @@
         <f>Revenue!$C$109</f>
         <v/>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="23">
+        <f>CHOOSE(Inputs!$B$4,B10,C10,D10)</f>
+        <v/>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>+4.05% (WS08)</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>WS08: ex-FX run-rate +3.25% plus FX +0.80pp; r 0.96, walk-forward 0.44x naive</t>
         </is>
@@ -19728,17 +20102,21 @@
         <f>Revenue!$C$107</f>
         <v/>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="27">
+        <f>CHOOSE(Inputs!$B$4,B11,C11,D11)</f>
+        <v/>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>+0.80pp</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>WS05 05_fx_schedule.csv broad-USD fit; WS08 refit</t>
         </is>
@@ -19762,17 +20140,21 @@
         <f>Revenue!$C$110</f>
         <v/>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="22">
+        <f>CHOOSE(Inputs!$B$4,B12,C12,D12)</f>
+        <v/>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>mid-teens growth</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>$26.6-27.2bn (WS02 cushion)</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>2Q26 letter; WS02</t>
         </is>
@@ -19796,17 +20178,21 @@
         <f>Revenue!$C$111</f>
         <v/>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="23">
+        <f>CHOOSE(Inputs!$B$4,B13,C13,D13)</f>
+        <v/>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>mid teens (14-16%)</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>16-19%</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>WS02</t>
         </is>
@@ -19830,17 +20216,21 @@
         <f>Revenue!$C$112</f>
         <v/>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="27">
+        <f>CHOOSE(Inputs!$B$4,B14,C14,D14)</f>
+        <v/>
+      </c>
+      <c r="F14" t="inlineStr">
         <is>
           <t>'relatively in line y/y'</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>17.9% +/- 0.2pt</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>2Q26 call; WS02. 3Q25 actual 17.88%</t>
         </is>
@@ -19864,17 +20254,21 @@
         <f>Revenue!$C$122</f>
         <v/>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="23">
+        <f>CHOOSE(Inputs!$B$4,B15,C15,D15)</f>
+        <v/>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>'down slightly' vs 50.1%</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>48.7-50.0%</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>WS07 5 Nov card (bear 48.3 / base 49.0 / bull 50.2); WS02 says 9 of 10 such ceilings were met</t>
         </is>
@@ -19898,17 +20292,21 @@
         <f>Revenue!$C$123</f>
         <v/>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="22">
+        <f>CHOOSE(Inputs!$B$4,B16,C16,D16)</f>
+        <v/>
+      </c>
+      <c r="F16" t="inlineStr">
         <is>
           <t>up y/y</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>$2,300-2,400m (derived)</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>WS04 04_q3_2026_breakeven.csv</t>
         </is>
@@ -19939,17 +20337,21 @@
         <f>Revenue!$D$118</f>
         <v/>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="22">
+        <f>CHOOSE(Inputs!$B$4,B19,C19,D19)</f>
+        <v/>
+      </c>
+      <c r="F19" t="inlineStr">
         <is>
           <t>no guide yet</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Street $3,200m (3,050-3,700)</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>WS04 Zacks 10 est - the widest spread in the table (21% high-low)</t>
         </is>
@@ -19973,17 +20375,21 @@
         <f>Revenue!$D$119</f>
         <v/>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="23">
+        <f>CHOOSE(Inputs!$B$4,B20,C20,D20)</f>
+        <v/>
+      </c>
+      <c r="F20" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>+11-13% expected</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>WS05: FX goes from about +3pp in Q3 to -0.4pp in Q4 and 84% of it is already realised</t>
         </is>
@@ -20007,17 +20413,21 @@
         <f>Revenue!$D$105</f>
         <v/>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="23">
+        <f>CHOOSE(Inputs!$B$4,B21,C21,D21)</f>
+        <v/>
+      </c>
+      <c r="F21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>accelerating vs Q3 is the bull tell</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>WS05: post-2022 an accelerating nights guide averaged +6.7% day-1 (n 5), a decelerating one -5.4% (n 9)</t>
         </is>
@@ -20041,17 +20451,21 @@
         <f>Revenue!$I$118</f>
         <v/>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="22">
+        <f>CHOOSE(Inputs!$B$4,B22,C22,D22)</f>
+        <v/>
+      </c>
+      <c r="F22" t="inlineStr">
         <is>
           <t>'at least mid teens' growth</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Street $14,100-14,160m</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>2Q26 letter; WS04</t>
         </is>
@@ -20075,17 +20489,21 @@
         <f>Revenue!$I$119</f>
         <v/>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="23">
+        <f>CHOOSE(Inputs!$B$4,B23,C23,D23)</f>
+        <v/>
+      </c>
+      <c r="F23" t="inlineStr">
         <is>
           <t>at least +14-16%</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>+15.2% to +15.6%</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>WS04</t>
         </is>
@@ -20109,17 +20527,21 @@
         <f>Costs!$D$82</f>
         <v/>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="23">
+        <f>CHOOSE(Inputs!$B$4,B24,C24,D24)</f>
+        <v/>
+      </c>
+      <c r="F24" t="inlineStr">
         <is>
           <t>'at least 35.5%'</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>36.1-36.9% on the FY24/FY25 cushion</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>WS02: FY24 beat the floor by 140bp, FY25 by 60bp</t>
         </is>
@@ -20141,7 +20563,7 @@
       <c r="C27" s="9" t="n">
         <v>-0.325</v>
       </c>
-      <c r="G27" s="17" t="inlineStr">
+      <c r="H27" s="17" t="inlineStr">
         <is>
           <t>WS08 08_demand_index_quarterly.csv, demand_eq; 2Q26 was -0.509, so the index improved. Only 4 of 7 components are populated for 3Q26 and no composite beat a naive baseline walk-forward.</t>
         </is>
@@ -20156,7 +20578,7 @@
       <c r="C28" s="20" t="n">
         <v>0.12</v>
       </c>
-      <c r="G28" s="17" t="inlineStr">
+      <c r="H28" s="17" t="inlineStr">
         <is>
           <t>WS08 08_backlog_tests.csv: funds held +10.46% y/y at 2Q26 x slope 0.60. Under-shot 1Q26 by 3.4pp and 2Q26 by 2.8pp because RNPL defers guest cash to check-in; add ~3pp.</t>
         </is>
@@ -20171,7 +20593,7 @@
       <c r="C29" s="20" t="n">
         <v>0.0707</v>
       </c>
-      <c r="G29" s="17" t="inlineStr">
+      <c r="H29" s="17" t="inlineStr">
         <is>
           <t>WS09, n 23; median 6.87%</t>
         </is>
@@ -20186,7 +20608,7 @@
       <c r="C30" s="20" t="n">
         <v>-0.037</v>
       </c>
-      <c r="G30" s="17" t="inlineStr">
+      <c r="H30" s="17" t="inlineStr">
         <is>
           <t>WS09, n 23, t -2.16</t>
         </is>
@@ -20201,7 +20623,7 @@
       <c r="C31" s="20" t="n">
         <v>0.8095238095238095</v>
       </c>
-      <c r="G31" s="17" t="inlineStr">
+      <c r="H31" s="17" t="inlineStr">
         <is>
           <t>WS01/predictive study: the sign of the nights-growth acceleration has set the day-1 direction in 17 of 21 prints</t>
         </is>
@@ -20216,7 +20638,7 @@
       <c r="C32" s="11" t="n">
         <v>0.97</v>
       </c>
-      <c r="G32" s="17" t="inlineStr">
+      <c r="H32" s="17" t="inlineStr">
         <is>
           <t>WS12: day-1 move correlates +0.97 with the change in the EV/NTM-revenue multiple, +0.09 with the estimate change</t>
         </is>
@@ -20231,7 +20653,7 @@
       <c r="C33" s="9" t="n">
         <v>9.109999999999999</v>
       </c>
-      <c r="G33" s="17" t="inlineStr">
+      <c r="H33" s="17" t="inlineStr">
         <is>
           <t>WS12: $9.11 per share = 5.0% at $181.94</t>
         </is>
@@ -20246,7 +20668,7 @@
       <c r="C34" s="20" t="n">
         <v>-0.051</v>
       </c>
-      <c r="G34" s="17" t="inlineStr">
+      <c r="H34" s="17" t="inlineStr">
         <is>
           <t>WS09: ABNB has underperformed in every November since 2021</t>
         </is>
@@ -20284,7 +20706,7 @@
     <row r="2">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>LibreOffice headless is not installed on this machine and the `formulas` package is not available, so the workbook is recalculated instead by a purpose-built evaluator, analysis/src/overnight/13_xlsx_eval.py, which walks the formula graph. Column D is also a live Excel formula, so Excel re-checks the same thing when the file is opened. Every |delta| should be 0.00. Full results: data/processed/overnight/13_reconciliation.csv.</t>
+          <t>Column B is the Python mirror (13_driver_model.py), column C is this workbook and column D is a live Excel formula, so Excel re-checks the difference every time the file is opened. Every |delta| should be 0.00. The same 216 outputs are also checked outside Excel by analysis/src/overnight/13_xlsx_eval.py. Workstream 17 then rebuilt the file in Excel 16.0 itself (Application.CalculateFullRebuild via COM): 0 error cells in 5,544, no circular reference, all 216 outputs and all 2,348 formula cells agreeing with the mirror to better than 1e-6 relative (worst 4.2e-15). Full results: data/processed/overnight/13_reconciliation.csv and 17_excel_vs_python.csv; the audit is research/notes/overnight/17_excel-audit.md.</t>
         </is>
       </c>
     </row>
@@ -20506,7 +20928,7 @@
         </is>
       </c>
       <c r="B13" s="15" t="n">
-        <v>580.4674837858635</v>
+        <v>589.0194789491042</v>
       </c>
       <c r="C13" s="15">
         <f>Cash!$D$23</f>
@@ -20529,7 +20951,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>7.846926841744251</v>
+        <v>7.732997026525528</v>
       </c>
       <c r="C14" s="9">
         <f>Cash!$D$24</f>
@@ -20759,7 +21181,7 @@
         </is>
       </c>
       <c r="B24" s="15" t="n">
-        <v>571.8773382119693</v>
+        <v>580.42933337521</v>
       </c>
       <c r="C24" s="15">
         <f>Cash!$E$23</f>
@@ -20782,7 +21204,7 @@
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>6.175004145495138</v>
+        <v>6.084022173102078</v>
       </c>
       <c r="C25" s="9">
         <f>Cash!$E$24</f>
@@ -21012,7 +21434,7 @@
         </is>
       </c>
       <c r="B35" s="15" t="n">
-        <v>564.5092321741711</v>
+        <v>573.0612273374118</v>
       </c>
       <c r="C35" s="15">
         <f>Cash!$F$23</f>
@@ -21035,7 +21457,7 @@
         </is>
       </c>
       <c r="B36" s="9" t="n">
-        <v>5.529798213290698</v>
+        <v>5.447275080826329</v>
       </c>
       <c r="C36" s="9">
         <f>Cash!$F$24</f>
@@ -21771,7 +22193,7 @@
         </is>
       </c>
       <c r="B68" s="9" t="n">
-        <v>37.78687590623652</v>
+        <v>37.23012737303444</v>
       </c>
       <c r="C68" s="9">
         <f>Valuation!$B$43</f>
@@ -21794,7 +22216,7 @@
         </is>
       </c>
       <c r="B69" s="9" t="n">
-        <v>110.0867420810157</v>
+        <v>108.4647336267925</v>
       </c>
       <c r="C69" s="9">
         <f>Valuation!$B$44</f>
@@ -21817,7 +22239,7 @@
         </is>
       </c>
       <c r="B70" s="9" t="n">
-        <v>77.08986621229708</v>
+        <v>75.95071074482665</v>
       </c>
       <c r="C70" s="9">
         <f>Valuation!$B$45</f>
@@ -21840,7 +22262,7 @@
         </is>
       </c>
       <c r="B71" s="9" t="n">
-        <v>110.0867420810157</v>
+        <v>108.4647336267925</v>
       </c>
       <c r="C71" s="9">
         <f>Valuation!$B$19</f>
@@ -21863,7 +22285,7 @@
         </is>
       </c>
       <c r="B72" s="9" t="n">
-        <v>84.80278774683526</v>
+        <v>83.55331087008436</v>
       </c>
       <c r="C72" s="9">
         <f>Valuation!$B$20</f>
@@ -21886,7 +22308,7 @@
         </is>
       </c>
       <c r="B73" s="9" t="n">
-        <v>37.78687590623652</v>
+        <v>37.23012737303444</v>
       </c>
       <c r="C73" s="9">
         <f>Valuation!$B$21</f>
@@ -21909,7 +22331,7 @@
         </is>
       </c>
       <c r="B74" s="9" t="n">
-        <v>46.01322689567024</v>
+        <v>45.33527202462913</v>
       </c>
       <c r="C74" s="9">
         <f>Valuation!$B$22</f>
@@ -21932,7 +22354,7 @@
         </is>
       </c>
       <c r="B75" s="9" t="n">
-        <v>105.155010468477</v>
+        <v>103.5857450950452</v>
       </c>
       <c r="C75" s="9">
         <f>Valuation!$B$23</f>
@@ -21955,7 +22377,7 @@
         </is>
       </c>
       <c r="B76" s="9" t="n">
-        <v>78.69455417554768</v>
+        <v>77.53507547937431</v>
       </c>
       <c r="C76" s="9">
         <f>Valuation!$B$39</f>
@@ -22162,7 +22584,7 @@
         </is>
       </c>
       <c r="B85" s="15" t="n">
-        <v>580.2980350665055</v>
+        <v>588.8500302297462</v>
       </c>
       <c r="C85" s="15">
         <f>Cash!$D$48</f>
@@ -22185,7 +22607,7 @@
         </is>
       </c>
       <c r="B86" s="9" t="n">
-        <v>8.838103930511778</v>
+        <v>8.709746253368642</v>
       </c>
       <c r="C86" s="9">
         <f>Cash!$D$49</f>
@@ -22415,7 +22837,7 @@
         </is>
       </c>
       <c r="B96" s="15" t="n">
-        <v>566.0461830692484</v>
+        <v>574.5981782324891</v>
       </c>
       <c r="C96" s="15">
         <f>Cash!$E$48</f>
@@ -22438,7 +22860,7 @@
         </is>
       </c>
       <c r="B97" s="9" t="n">
-        <v>9.575812439782297</v>
+        <v>9.433291448990044</v>
       </c>
       <c r="C97" s="9">
         <f>Cash!$E$49</f>
@@ -22668,7 +23090,7 @@
         </is>
       </c>
       <c r="B107" s="15" t="n">
-        <v>552.9824383296977</v>
+        <v>561.5344334929384</v>
       </c>
       <c r="C107" s="15">
         <f>Cash!$F$48</f>
@@ -22691,7 +23113,7 @@
         </is>
       </c>
       <c r="B108" s="9" t="n">
-        <v>11.2069485180663</v>
+        <v>11.03627016994609</v>
       </c>
       <c r="C108" s="9">
         <f>Cash!$F$49</f>
@@ -23427,7 +23849,7 @@
         </is>
       </c>
       <c r="B140" s="9" t="n">
-        <v>112.2504385986892</v>
+        <v>110.5797663892496</v>
       </c>
       <c r="C140" s="9">
         <f>Valuation!$C$43</f>
@@ -23450,7 +23872,7 @@
         </is>
       </c>
       <c r="B141" s="9" t="n">
-        <v>220.8753904700754</v>
+        <v>217.5115268166406</v>
       </c>
       <c r="C141" s="9">
         <f>Valuation!$C$44</f>
@@ -23473,7 +23895,7 @@
         </is>
       </c>
       <c r="B142" s="9" t="n">
-        <v>162.6527676055112</v>
+        <v>160.2191890732878</v>
       </c>
       <c r="C142" s="9">
         <f>Valuation!$C$45</f>
@@ -23496,7 +23918,7 @@
         </is>
       </c>
       <c r="B143" s="9" t="n">
-        <v>183.6090265557019</v>
+        <v>180.8762933753395</v>
       </c>
       <c r="C143" s="9">
         <f>Valuation!$C$19</f>
@@ -23519,7 +23941,7 @@
         </is>
       </c>
       <c r="B144" s="9" t="n">
-        <v>154.8054280018954</v>
+        <v>152.5013913347621</v>
       </c>
       <c r="C144" s="9">
         <f>Valuation!$C$20</f>
@@ -23542,7 +23964,7 @@
         </is>
       </c>
       <c r="B145" s="9" t="n">
-        <v>119.0287985346427</v>
+        <v>117.25724103948</v>
       </c>
       <c r="C145" s="9">
         <f>Valuation!$C$21</f>
@@ -23565,7 +23987,7 @@
         </is>
       </c>
       <c r="B146" s="9" t="n">
-        <v>112.2504385986892</v>
+        <v>110.5797663892496</v>
       </c>
       <c r="C146" s="9">
         <f>Valuation!$C$22</f>
@@ -23588,7 +24010,7 @@
         </is>
       </c>
       <c r="B147" s="9" t="n">
-        <v>220.8753904700754</v>
+        <v>217.5115268166406</v>
       </c>
       <c r="C147" s="9">
         <f>Valuation!$C$23</f>
@@ -23611,7 +24033,7 @@
         </is>
       </c>
       <c r="B148" s="9" t="n">
-        <v>185.3475234720625</v>
+        <v>182.5889154842552</v>
       </c>
       <c r="C148" s="9">
         <f>Valuation!$C$39</f>
@@ -23818,7 +24240,7 @@
         </is>
       </c>
       <c r="B157" s="15" t="n">
-        <v>580.1285863471475</v>
+        <v>588.680581510388</v>
       </c>
       <c r="C157" s="15">
         <f>Cash!$D$73</f>
@@ -23841,7 +24263,7 @@
         </is>
       </c>
       <c r="B158" s="9" t="n">
-        <v>9.756249727354881</v>
+        <v>9.614516836717254</v>
       </c>
       <c r="C158" s="9">
         <f>Cash!$D$74</f>
@@ -24071,7 +24493,7 @@
         </is>
       </c>
       <c r="B168" s="15" t="n">
-        <v>562.8452323371913</v>
+        <v>571.3972275004319</v>
       </c>
       <c r="C168" s="15">
         <f>Cash!$E$73</f>
@@ -24094,7 +24516,7 @@
         </is>
       </c>
       <c r="B169" s="9" t="n">
-        <v>11.62535732632006</v>
+        <v>11.4513627830484</v>
       </c>
       <c r="C169" s="9">
         <f>Cash!$E$74</f>
@@ -24324,7 +24746,7 @@
         </is>
       </c>
       <c r="B179" s="15" t="n">
-        <v>546.6238396526029</v>
+        <v>555.1758348158435</v>
       </c>
       <c r="C179" s="15">
         <f>Cash!$F$73</f>
@@ -24347,7 +24769,7 @@
         </is>
       </c>
       <c r="B180" s="9" t="n">
-        <v>13.89001990477269</v>
+        <v>13.67605637179159</v>
       </c>
       <c r="C180" s="9">
         <f>Cash!$F$74</f>
@@ -25083,7 +25505,7 @@
         </is>
       </c>
       <c r="B212" s="9" t="n">
-        <v>179.1737878590949</v>
+        <v>176.4921273724778</v>
       </c>
       <c r="C212" s="9">
         <f>Valuation!$D$43</f>
@@ -25106,7 +25528,7 @@
         </is>
       </c>
       <c r="B213" s="9" t="n">
-        <v>293.6145528813599</v>
+        <v>289.0916790842117</v>
       </c>
       <c r="C213" s="9">
         <f>Valuation!$D$44</f>
@@ -25129,7 +25551,7 @@
         </is>
       </c>
       <c r="B214" s="9" t="n">
-        <v>236.2390078668021</v>
+        <v>232.6818629592952</v>
       </c>
       <c r="C214" s="9">
         <f>Valuation!$D$45</f>
@@ -25152,7 +25574,7 @@
         </is>
       </c>
       <c r="B215" s="9" t="n">
-        <v>237.7142133420388</v>
+        <v>234.1563892839354</v>
       </c>
       <c r="C215" s="9">
         <f>Valuation!$D$19</f>
@@ -25175,7 +25597,7 @@
         </is>
       </c>
       <c r="B216" s="9" t="n">
-        <v>221.2472438381016</v>
+        <v>217.9358778248979</v>
       </c>
       <c r="C216" s="9">
         <f>Valuation!$D$20</f>
@@ -25198,7 +25620,7 @@
         </is>
       </c>
       <c r="B217" s="9" t="n">
-        <v>200.4031236431927</v>
+        <v>197.4037276685358</v>
       </c>
       <c r="C217" s="9">
         <f>Valuation!$D$21</f>
@@ -25221,7 +25643,7 @@
         </is>
       </c>
       <c r="B218" s="9" t="n">
-        <v>179.1737878590949</v>
+        <v>176.4921273724778</v>
       </c>
       <c r="C218" s="9">
         <f>Valuation!$D$22</f>
@@ -25244,7 +25666,7 @@
         </is>
       </c>
       <c r="B219" s="9" t="n">
-        <v>293.6145528813599</v>
+        <v>289.0916790842117</v>
       </c>
       <c r="C219" s="9">
         <f>Valuation!$D$23</f>
@@ -25267,7 +25689,7 @@
         </is>
       </c>
       <c r="B220" s="9" t="n">
-        <v>285.2811256370247</v>
+        <v>281.0113765217127</v>
       </c>
       <c r="C220" s="9">
         <f>Valuation!$D$39</f>

</xml_diff>